<commit_message>
33 more Ledger stamps, and Try it follows the bust setting
Every chapter now has at least 10 stamps (12 for most): drop totals, every
Demonlord and lava drop, corpse items, Inquisitor kills, Dwarven O's, a 10M drop
and the Ghosts' and sharks' runs of luck. Added to docs/ledger_stamps.xlsx and
regenerated; LedgerTest covers them (388 checks).

The menu's Try it now shortens busts when Busts is Short and plays nothing (with
a chat note) when it is None. /butcher test still plays everything in full.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E2z82eUcdf81sbDmiwVwoi
</commit_message>
<xml_diff>
--- a/docs/ledger_stamps.xlsx
+++ b/docs/ledger_stamps.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stamps'!$A$1:$M$90</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stamps'!$A$1:$M$140</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
 </workbook>
@@ -407,7 +407,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M90"/>
+  <dimension ref="A1:M140"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -936,22 +936,22 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>scatha_worm_food</t>
+          <t>house_well_done</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Scatha</t>
+          <t>House</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Worm Food</t>
+          <t>Well Done</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Scatha kills</t>
+          <t>Rare drops revealed, every animation together</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -960,16 +960,16 @@
         </is>
       </c>
       <c r="F11" s="4" t="n">
-        <v>50</v>
+        <v>5</v>
       </c>
       <c r="G11" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="H11" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="H11" s="4" t="n">
-        <v>500</v>
-      </c>
       <c r="I11" s="4" t="n">
-        <v>1000</v>
+        <v>250</v>
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
@@ -986,38 +986,50 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="M11" s="3" t="n"/>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>scatha_rare_cut</t>
+          <t>house_collector</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Scatha</t>
+          <t>House</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Rare Cut</t>
+          <t>Collector</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>A rare Scatha pet</t>
+          <t>Rare drops from different animations</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Single</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="n"/>
-      <c r="G12" s="4" t="n"/>
-      <c r="H12" s="4" t="n"/>
-      <c r="I12" s="4" t="n"/>
+          <t>Tiered</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>7</v>
+      </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
           <t>No</t>
@@ -1033,27 +1045,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="M12" s="3" t="n"/>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>scatha_choice_cut</t>
+          <t>house_big_ticket</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Scatha</t>
+          <t>House</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Choice Cut</t>
+          <t>Big Ticket</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>An epic Scatha pet</t>
+          <t>A single drop worth 10,000,000 coins or more</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -1072,7 +1088,7 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L13" s="3" t="inlineStr">
@@ -1080,12 +1096,16 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="M13" s="3" t="n"/>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>scatha_prime_cut</t>
+          <t>scatha_worm_food</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -1095,23 +1115,31 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Prime Cut</t>
+          <t>Worm Food</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>A legendary Scatha pet</t>
+          <t>Scatha kills</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Single</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="n"/>
-      <c r="G14" s="4" t="n"/>
-      <c r="H14" s="4" t="n"/>
-      <c r="I14" s="4" t="n"/>
+          <t>Tiered</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="H14" s="4" t="n">
+        <v>500</v>
+      </c>
+      <c r="I14" s="4" t="n">
+        <v>1000</v>
+      </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
           <t>No</t>
@@ -1132,7 +1160,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>scatha_full_set</t>
+          <t>scatha_rare_cut</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1142,12 +1170,12 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Full Set</t>
+          <t>Rare Cut</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>All three pet rarities</t>
+          <t>A rare Scatha pet</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
@@ -1179,7 +1207,7 @@
     <row r="16" ht="28.5" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>scatha_beginners_luck</t>
+          <t>scatha_choice_cut</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1189,12 +1217,12 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Beginner's Luck</t>
+          <t>Choice Cut</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>A pet within your first N kills</t>
+          <t>An epic Scatha pet</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -1202,9 +1230,7 @@
           <t>Single</t>
         </is>
       </c>
-      <c r="F16" s="4" t="n">
-        <v>20</v>
-      </c>
+      <c r="F16" s="4" t="n"/>
       <c r="G16" s="4" t="n"/>
       <c r="H16" s="4" t="n"/>
       <c r="I16" s="4" t="n"/>
@@ -1215,7 +1241,7 @@
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Partly</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="L16" s="3" t="inlineStr">
@@ -1228,7 +1254,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>scatha_dry_aged</t>
+          <t>scatha_prime_cut</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1238,12 +1264,12 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Dry Aged</t>
+          <t>Prime Cut</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Kills in a row without a pet</t>
+          <t>A legendary Scatha pet</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
@@ -1251,9 +1277,7 @@
           <t>Single</t>
         </is>
       </c>
-      <c r="F17" s="4" t="n">
-        <v>100</v>
-      </c>
+      <c r="F17" s="4" t="n"/>
       <c r="G17" s="4" t="n"/>
       <c r="H17" s="4" t="n"/>
       <c r="I17" s="4" t="n"/>
@@ -1277,7 +1301,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>scatha_dry_aged_45</t>
+          <t>scatha_full_set</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -1287,12 +1311,12 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Dry Aged 45 Days</t>
+          <t>Full Set</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Kills in a row without a pet</t>
+          <t>All three pet rarities</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -1300,15 +1324,13 @@
           <t>Single</t>
         </is>
       </c>
-      <c r="F18" s="4" t="n">
-        <v>200</v>
-      </c>
+      <c r="F18" s="4" t="n"/>
       <c r="G18" s="4" t="n"/>
       <c r="H18" s="4" t="n"/>
       <c r="I18" s="4" t="n"/>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1326,7 +1348,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>scatha_slippery</t>
+          <t>scatha_beginners_luck</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1336,12 +1358,12 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Slippery</t>
+          <t>Beginner's Luck</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Times the Scatha ducks your last swing</t>
+          <t>A pet within your first N kills</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
@@ -1350,7 +1372,7 @@
         </is>
       </c>
       <c r="F19" s="4" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="G19" s="4" t="n"/>
       <c r="H19" s="4" t="n"/>
@@ -1362,7 +1384,7 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Partly</t>
         </is>
       </c>
       <c r="L19" s="3" t="inlineStr">
@@ -1375,7 +1397,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>scatha_back_to_back</t>
+          <t>scatha_dry_aged</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1385,12 +1407,12 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Back to Back</t>
+          <t>Dry Aged</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Two pets within N kills</t>
+          <t>Kills in a row without a pet</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
@@ -1399,7 +1421,7 @@
         </is>
       </c>
       <c r="F20" s="4" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="G20" s="4" t="n"/>
       <c r="H20" s="4" t="n"/>
@@ -1411,7 +1433,7 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="L20" s="3" t="inlineStr">
@@ -1424,7 +1446,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>scatha_dozen</t>
+          <t>scatha_dry_aged_45</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1434,12 +1456,12 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>A Butcher's Dozen</t>
+          <t>Dry Aged 45 Days</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Pets in total</t>
+          <t>Kills in a row without a pet</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
@@ -1448,14 +1470,14 @@
         </is>
       </c>
       <c r="F21" s="4" t="n">
-        <v>13</v>
+        <v>200</v>
       </c>
       <c r="G21" s="4" t="n"/>
       <c r="H21" s="4" t="n"/>
       <c r="I21" s="4" t="n"/>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -1473,41 +1495,35 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>vg_thawed_out</t>
+          <t>scatha_slippery</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Vanguard</t>
+          <t>Scatha</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Thawed Out</t>
+          <t>Slippery</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Vanguard corpses opened</t>
+          <t>Times the Scatha ducks your last swing</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Tiered</t>
+          <t>Single</t>
         </is>
       </c>
       <c r="F22" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="G22" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="H22" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="I22" s="4" t="n">
-        <v>100</v>
-      </c>
+      <c r="G22" s="4" t="n"/>
+      <c r="H22" s="4" t="n"/>
+      <c r="I22" s="4" t="n"/>
       <c r="J22" s="3" t="inlineStr">
         <is>
           <t>No</t>
@@ -1528,22 +1544,22 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>vg_cold_hands</t>
+          <t>scatha_back_to_back</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Vanguard</t>
+          <t>Scatha</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Cold Hands</t>
+          <t>Back to Back</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>A legendary drop</t>
+          <t>Two pets within N kills</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
@@ -1551,7 +1567,9 @@
           <t>Single</t>
         </is>
       </c>
-      <c r="F23" s="4" t="n"/>
+      <c r="F23" s="4" t="n">
+        <v>50</v>
+      </c>
       <c r="G23" s="4" t="n"/>
       <c r="H23" s="4" t="n"/>
       <c r="I23" s="4" t="n"/>
@@ -1562,7 +1580,7 @@
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L23" s="3" t="inlineStr">
@@ -1575,22 +1593,22 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>vg_heart_of_glass</t>
+          <t>scatha_dozen</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Vanguard</t>
+          <t>Scatha</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Heart of Glass</t>
+          <t>A Butcher's Dozen</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>The Shattered Locket</t>
+          <t>Pets in total</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
@@ -1598,7 +1616,9 @@
           <t>Single</t>
         </is>
       </c>
-      <c r="F24" s="4" t="n"/>
+      <c r="F24" s="4" t="n">
+        <v>13</v>
+      </c>
       <c r="G24" s="4" t="n"/>
       <c r="H24" s="4" t="n"/>
       <c r="I24" s="4" t="n"/>
@@ -1622,33 +1642,41 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>vg_frostbitten</t>
+          <t>scatha_cereal</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Vanguard</t>
+          <t>Scatha</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Frostbitten</t>
+          <t>Part of a Balanced Breakfast</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>The Frostbitten Dye</t>
+          <t>Busts that were Dwarven O's</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Single</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="n"/>
-      <c r="G25" s="4" t="n"/>
-      <c r="H25" s="4" t="n"/>
-      <c r="I25" s="4" t="n"/>
+          <t>Tiered</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="H25" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="I25" s="4" t="n">
+        <v>250</v>
+      </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
           <t>No</t>
@@ -1664,12 +1692,16 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="M25" s="3" t="n"/>
+      <c r="M25" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>vg_ice_cold</t>
+          <t>vg_thawed_out</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1679,25 +1711,31 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Ice Cold</t>
+          <t>Thawed Out</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Corpses in a row without a legendary</t>
+          <t>Vanguard corpses opened</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Single</t>
+          <t>Tiered</t>
         </is>
       </c>
       <c r="F26" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G26" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="G26" s="4" t="n"/>
-      <c r="H26" s="4" t="n"/>
-      <c r="I26" s="4" t="n"/>
+      <c r="H26" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="I26" s="4" t="n">
+        <v>100</v>
+      </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
           <t>No</t>
@@ -1713,16 +1751,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="M26" s="3" t="inlineStr">
-        <is>
-          <t>Claude: was 'nothing above common'. Your stats count corpses since a legendary, so this way it can be backfilled.</t>
-        </is>
-      </c>
+      <c r="M26" s="3" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>vg_negative_equity</t>
+          <t>vg_cold_hands</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1732,12 +1766,12 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Negative Equity</t>
+          <t>Cold Hands</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>A corpse worth less than its Skeleton Key</t>
+          <t>A legendary drop</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
@@ -1756,7 +1790,7 @@
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="L27" s="3" t="inlineStr">
@@ -1769,7 +1803,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>vg_in_the_black</t>
+          <t>vg_heart_of_glass</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1779,12 +1813,12 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>In the Black</t>
+          <t>Heart of Glass</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>A corpse worth at least N coins</t>
+          <t>The Shattered Locket</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
@@ -1792,9 +1826,7 @@
           <t>Single</t>
         </is>
       </c>
-      <c r="F28" s="4" t="n">
-        <v>30000000</v>
-      </c>
+      <c r="F28" s="4" t="n"/>
       <c r="G28" s="4" t="n"/>
       <c r="H28" s="4" t="n"/>
       <c r="I28" s="4" t="n"/>
@@ -1805,7 +1837,7 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="L28" s="3" t="inlineStr">
@@ -1818,41 +1850,33 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>diana_heads</t>
+          <t>vg_frostbitten</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Diana</t>
+          <t>Vanguard</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Off With Their Heads</t>
+          <t>Frostbitten</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Diana creature kills</t>
+          <t>The Frostbitten Dye</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Tiered</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="G29" s="4" t="n">
-        <v>250</v>
-      </c>
-      <c r="H29" s="4" t="n">
-        <v>1000</v>
-      </c>
-      <c r="I29" s="4" t="n">
-        <v>5000</v>
-      </c>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="n"/>
+      <c r="G29" s="4" t="n"/>
+      <c r="H29" s="4" t="n"/>
+      <c r="I29" s="4" t="n"/>
       <c r="J29" s="3" t="inlineStr">
         <is>
           <t>No</t>
@@ -1873,22 +1897,22 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>diana_brain_food</t>
+          <t>vg_ice_cold</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Diana</t>
+          <t>Vanguard</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Food for Thought</t>
+          <t>Ice Cold</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Brain Food</t>
+          <t>Corpses in a row without a legendary</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
@@ -1896,7 +1920,9 @@
           <t>Single</t>
         </is>
       </c>
-      <c r="F30" s="4" t="n"/>
+      <c r="F30" s="4" t="n">
+        <v>25</v>
+      </c>
       <c r="G30" s="4" t="n"/>
       <c r="H30" s="4" t="n"/>
       <c r="I30" s="4" t="n"/>
@@ -1915,27 +1941,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="M30" s="3" t="n"/>
+      <c r="M30" s="3" t="inlineStr">
+        <is>
+          <t>Claude: was 'nothing above common'. Your stats count corpses since a legendary, so this way it can be backfilled.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>diana_chimera</t>
+          <t>vg_negative_equity</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Diana</t>
+          <t>Vanguard</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Glint in the Eye</t>
+          <t>Negative Equity</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Chimera I</t>
+          <t>A corpse worth less than its Skeleton Key</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
@@ -1954,7 +1984,7 @@
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L31" s="3" t="inlineStr">
@@ -1967,22 +1997,22 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>diana_stinger</t>
+          <t>vg_in_the_black</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Diana</t>
+          <t>Vanguard</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Sting Operation</t>
+          <t>In the Black</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Fateful Stinger</t>
+          <t>A corpse worth at least N coins</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -1990,7 +2020,9 @@
           <t>Single</t>
         </is>
       </c>
-      <c r="F32" s="4" t="n"/>
+      <c r="F32" s="4" t="n">
+        <v>30000000</v>
+      </c>
       <c r="G32" s="4" t="n"/>
       <c r="H32" s="4" t="n"/>
       <c r="I32" s="4" t="n"/>
@@ -2001,7 +2033,7 @@
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L32" s="3" t="inlineStr">
@@ -2014,33 +2046,41 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>diana_manticore</t>
+          <t>vg_skeleton_crew</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Diana</t>
+          <t>Vanguard</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Heart of the Beast</t>
+          <t>Skeleton Crew</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Manti-core</t>
+          <t>Loot rolled from corpses</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Single</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="n"/>
-      <c r="G33" s="4" t="n"/>
-      <c r="H33" s="4" t="n"/>
-      <c r="I33" s="4" t="n"/>
+          <t>Tiered</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="G33" s="4" t="n">
+        <v>500</v>
+      </c>
+      <c r="H33" s="4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I33" s="4" t="n">
+        <v>2500</v>
+      </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
           <t>No</t>
@@ -2056,38 +2096,50 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="M33" s="3" t="n"/>
+      <c r="M33" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>diana_crown</t>
+          <t>vg_cold_storage</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Diana</t>
+          <t>Vanguard</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Greed is Good</t>
+          <t>Cold Storage</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Crown of Greed</t>
+          <t>Legendary drops in total</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Single</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="n"/>
-      <c r="G34" s="4" t="n"/>
-      <c r="H34" s="4" t="n"/>
-      <c r="I34" s="4" t="n"/>
+          <t>Tiered</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G34" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="H34" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="I34" s="4" t="n">
+        <v>50</v>
+      </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
           <t>No</t>
@@ -2103,27 +2155,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="M34" s="3" t="n"/>
+      <c r="M34" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>diana_wool</t>
+          <t>vg_will_o_wisp</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Diana</t>
+          <t>Vanguard</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Golden Fleece</t>
+          <t>Will-o'-the-Wisp</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Shimmering Wool</t>
+          <t>A Caged Wisp</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
@@ -2150,27 +2206,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="M35" s="3" t="n"/>
+      <c r="M35" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>diana_relic</t>
+          <t>vg_tough_skin</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Diana</t>
+          <t>Vanguard</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Relic Hunter</t>
+          <t>Tough Skin</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Minos Relic</t>
+          <t>A Frozen Scute</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
@@ -2197,27 +2257,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="M36" s="3" t="n"/>
+      <c r="M36" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>diana_dye</t>
+          <t>vg_master_key</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Diana</t>
+          <t>Vanguard</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>The Whole Hunt</t>
+          <t>Master Key</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Mythological Dye</t>
+          <t>A Skeleton Key from a corpse</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
@@ -2244,12 +2308,16 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="M37" s="3" t="n"/>
+      <c r="M37" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>diana_pantheon</t>
+          <t>diana_heads</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -2259,23 +2327,31 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Pantheon</t>
+          <t>Off With Their Heads</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>All eight Diana drops</t>
+          <t>Diana creature kills</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Single</t>
-        </is>
-      </c>
-      <c r="F38" s="4" t="n"/>
-      <c r="G38" s="4" t="n"/>
-      <c r="H38" s="4" t="n"/>
-      <c r="I38" s="4" t="n"/>
+          <t>Tiered</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="G38" s="4" t="n">
+        <v>250</v>
+      </c>
+      <c r="H38" s="4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I38" s="4" t="n">
+        <v>5000</v>
+      </c>
       <c r="J38" s="3" t="inlineStr">
         <is>
           <t>No</t>
@@ -2296,7 +2372,7 @@
     <row r="39" ht="28.5" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>diana_shared_custody</t>
+          <t>diana_brain_food</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -2306,12 +2382,12 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Shared Custody</t>
+          <t>Food for Thought</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>A win from loot share</t>
+          <t>Brain Food</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
@@ -2325,12 +2401,12 @@
       <c r="I39" s="4" t="n"/>
       <c r="J39" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="L39" s="3" t="inlineStr">
@@ -2343,41 +2419,33 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>hellion_fire_watch</t>
+          <t>diana_chimera</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Hellion</t>
+          <t>Diana</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Fire Watch</t>
+          <t>Glint in the Eye</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>Tier IV Demonlords killed</t>
+          <t>Chimera I</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Tiered</t>
-        </is>
-      </c>
-      <c r="F40" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="G40" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="H40" s="4" t="n">
-        <v>500</v>
-      </c>
-      <c r="I40" s="4" t="n">
-        <v>1000</v>
-      </c>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="n"/>
+      <c r="G40" s="4" t="n"/>
+      <c r="H40" s="4" t="n"/>
+      <c r="I40" s="4" t="n"/>
       <c r="J40" s="3" t="inlineStr">
         <is>
           <t>No</t>
@@ -2398,22 +2466,22 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>hellion_double_down</t>
+          <t>diana_stinger</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Hellion</t>
+          <t>Diana</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Double Down</t>
+          <t>Sting Operation</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Duplex I</t>
+          <t>Fateful Stinger</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
@@ -2445,22 +2513,22 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>hellion_roll_dice</t>
+          <t>diana_manticore</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Hellion</t>
+          <t>Diana</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Roll the Dice</t>
+          <t>Heart of the Beast</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>Archfiend Dice</t>
+          <t>Manti-core</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
@@ -2492,22 +2560,22 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>hellion_high_roller</t>
+          <t>diana_crown</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Hellion</t>
+          <t>Diana</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>High Roller</t>
+          <t>Greed is Good</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>High Class Archfiend Dice</t>
+          <t>Crown of Greed</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
@@ -2539,22 +2607,22 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>hellion_playing_fire</t>
+          <t>diana_wool</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>Hellion</t>
+          <t>Diana</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Playing With Fire</t>
+          <t>Golden Fleece</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Flame Dye</t>
+          <t>Shimmering Wool</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
@@ -2586,22 +2654,22 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>hellion_ashes</t>
+          <t>diana_relic</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Hellion</t>
+          <t>Diana</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Ashes to Ashes</t>
+          <t>Relic Hunter</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Bosses in a row that land on grey (busts)</t>
+          <t>Minos Relic</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
@@ -2609,9 +2677,7 @@
           <t>Single</t>
         </is>
       </c>
-      <c r="F45" s="4" t="n">
-        <v>25</v>
-      </c>
+      <c r="F45" s="4" t="n"/>
       <c r="G45" s="4" t="n"/>
       <c r="H45" s="4" t="n"/>
       <c r="I45" s="4" t="n"/>
@@ -2622,7 +2688,7 @@
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>Partly</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="L45" s="3" t="inlineStr">
@@ -2635,41 +2701,33 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>lava_magma_maker</t>
+          <t>diana_dye</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>Eruption</t>
+          <t>Diana</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Magma Maker</t>
+          <t>The Whole Hunt</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Rare lava creatures killed</t>
+          <t>Mythological Dye</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>Tiered</t>
-        </is>
-      </c>
-      <c r="F46" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="G46" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="H46" s="4" t="n">
-        <v>500</v>
-      </c>
-      <c r="I46" s="4" t="n">
-        <v>1000</v>
-      </c>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="n"/>
+      <c r="G46" s="4" t="n"/>
+      <c r="H46" s="4" t="n"/>
+      <c r="I46" s="4" t="n"/>
       <c r="J46" s="3" t="inlineStr">
         <is>
           <t>No</t>
@@ -2690,22 +2748,22 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>lava_flash</t>
+          <t>diana_pantheon</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Eruption</t>
+          <t>Diana</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>In a Flash</t>
+          <t>Pantheon</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Flash I</t>
+          <t>All eight Diana drops</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
@@ -2737,22 +2795,22 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>lava_meltdown</t>
+          <t>diana_shared_custody</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>Eruption</t>
+          <t>Diana</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Meltdown</t>
+          <t>Shared Custody</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Radioactive Vial</t>
+          <t>A win from loot share</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
@@ -2766,12 +2824,12 @@
       <c r="I48" s="4" t="n"/>
       <c r="J48" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L48" s="3" t="inlineStr">
@@ -2784,33 +2842,41 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>lava_end_times</t>
+          <t>diana_inquisition</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Eruption</t>
+          <t>Diana</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>End Times</t>
+          <t>The Inquisition</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Burnt Texts</t>
+          <t>Minos Inquisitor kills</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Single</t>
-        </is>
-      </c>
-      <c r="F49" s="4" t="n"/>
-      <c r="G49" s="4" t="n"/>
-      <c r="H49" s="4" t="n"/>
-      <c r="I49" s="4" t="n"/>
+          <t>Tiered</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="G49" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="H49" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="I49" s="4" t="n">
+        <v>250</v>
+      </c>
       <c r="J49" s="3" t="inlineStr">
         <is>
           <t>No</t>
@@ -2826,38 +2892,50 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="M49" s="3" t="n"/>
+      <c r="M49" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>lava_kuudra</t>
+          <t>hellion_fire_watch</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>Eruption</t>
+          <t>Hellion</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Kuudra Rises</t>
+          <t>Fire Watch</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>Carmine Dye</t>
+          <t>Tier IV Demonlords killed</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>Single</t>
-        </is>
-      </c>
-      <c r="F50" s="4" t="n"/>
-      <c r="G50" s="4" t="n"/>
-      <c r="H50" s="4" t="n"/>
-      <c r="I50" s="4" t="n"/>
+          <t>Tiered</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="G50" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="H50" s="4" t="n">
+        <v>500</v>
+      </c>
+      <c r="I50" s="4" t="n">
+        <v>1000</v>
+      </c>
       <c r="J50" s="3" t="inlineStr">
         <is>
           <t>No</t>
@@ -2878,22 +2956,22 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>lava_jaw_dropping</t>
+          <t>hellion_double_down</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Eruption</t>
+          <t>Hellion</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Jaw Dropping</t>
+          <t>Double Down</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Any win from a Lord Jawbus</t>
+          <t>Duplex I</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
@@ -2912,7 +2990,7 @@
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="L51" s="3" t="inlineStr">
@@ -2925,22 +3003,22 @@
     <row r="52" ht="28.5" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>lava_thermal_runaway</t>
+          <t>hellion_roll_dice</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>Eruption</t>
+          <t>Hellion</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Thermal Runaway</t>
+          <t>Roll the Dice</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Kills in a row with no win</t>
+          <t>Archfiend Dice</t>
         </is>
       </c>
       <c r="E52" s="3" t="inlineStr">
@@ -2948,9 +3026,7 @@
           <t>Single</t>
         </is>
       </c>
-      <c r="F52" s="4" t="n">
-        <v>50</v>
-      </c>
+      <c r="F52" s="4" t="n"/>
       <c r="G52" s="4" t="n"/>
       <c r="H52" s="4" t="n"/>
       <c r="I52" s="4" t="n"/>
@@ -2961,7 +3037,7 @@
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>Partly</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="L52" s="3" t="inlineStr">
@@ -2974,38 +3050,32 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>fin_shark_week</t>
+          <t>hellion_high_roller</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Fin</t>
+          <t>Hellion</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Shark Week</t>
+          <t>High Roller</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Great White Sharks killed</t>
+          <t>High Class Archfiend Dice</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>Tiered</t>
-        </is>
-      </c>
-      <c r="F53" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="G53" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="H53" s="4" t="n">
-        <v>500</v>
-      </c>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="n"/>
+      <c r="G53" s="4" t="n"/>
+      <c r="H53" s="4" t="n"/>
       <c r="I53" s="4" t="n"/>
       <c r="J53" s="3" t="inlineStr">
         <is>
@@ -3027,22 +3097,22 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>fin_big_fish</t>
+          <t>hellion_playing_fire</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>Fin</t>
+          <t>Hellion</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Big Fish</t>
+          <t>Playing With Fire</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>A Megalodon (any rarity)</t>
+          <t>Flame Dye</t>
         </is>
       </c>
       <c r="E54" s="3" t="inlineStr">
@@ -3069,31 +3139,27 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="M54" s="3" t="inlineStr">
-        <is>
-          <t>Claude: was 'Epic Megalodon'. The stats never kept the pet's rarity, so any Megalodon counts; Bigger Fish stays legendary-only, counted from the update.</t>
-        </is>
-      </c>
+      <c r="M54" s="3" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>fin_bigger_fish</t>
+          <t>hellion_ashes</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>Fin</t>
+          <t>Hellion</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Bigger Fish</t>
+          <t>Ashes to Ashes</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Legendary Megalodon</t>
+          <t>Bosses in a row that land on grey (busts)</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
@@ -3101,7 +3167,9 @@
           <t>Single</t>
         </is>
       </c>
-      <c r="F55" s="4" t="n"/>
+      <c r="F55" s="4" t="n">
+        <v>25</v>
+      </c>
       <c r="G55" s="4" t="n"/>
       <c r="H55" s="4" t="n"/>
       <c r="I55" s="4" t="n"/>
@@ -3112,7 +3180,7 @@
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Partly</t>
         </is>
       </c>
       <c r="L55" s="3" t="inlineStr">
@@ -3125,22 +3193,22 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>fin_tooth_fairy</t>
+          <t>hellion_power_trip</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>Fin</t>
+          <t>Hellion</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>Tooth Fairy</t>
+          <t>Power Trip</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>Great White Shark Tooth</t>
+          <t>Scorched Power Crystal</t>
         </is>
       </c>
       <c r="E56" s="3" t="inlineStr">
@@ -3167,27 +3235,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="M56" s="3" t="n"/>
+      <c r="M56" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>fin_off_the_hook</t>
+          <t>hellion_cold_feet</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>Fin</t>
+          <t>Hellion</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Off the Hook</t>
+          <t>Cold Feet</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>Sharks that dropped neither</t>
+          <t>Subzero Inverter</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
@@ -3195,9 +3267,7 @@
           <t>Single</t>
         </is>
       </c>
-      <c r="F57" s="4" t="n">
-        <v>50</v>
-      </c>
+      <c r="F57" s="4" t="n"/>
       <c r="G57" s="4" t="n"/>
       <c r="H57" s="4" t="n"/>
       <c r="I57" s="4" t="n"/>
@@ -3216,27 +3286,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="M57" s="3" t="n"/>
+      <c r="M57" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>wisp_sorrowful</t>
+          <t>hellion_blueprints</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>Wisp</t>
+          <t>Hellion</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>Sorrowful</t>
+          <t>Blueprints</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Sorrow</t>
+          <t>Wilson's Engineering Plans</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
@@ -3263,27 +3337,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="M58" s="3" t="n"/>
+      <c r="M58" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>wisp_plasma</t>
+          <t>hellion_paragon</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>Wisp</t>
+          <t>Hellion</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Plasma Screen</t>
+          <t>Paragon of Virtue</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>Plasma</t>
+          <t>Paragon Shard</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
@@ -3310,27 +3388,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="M59" s="3" t="n"/>
+      <c r="M59" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>wisp_spirit_level</t>
+          <t>hellion_hellfire_club</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>Wisp</t>
+          <t>Hellion</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>Spirit Level</t>
+          <t>Hellfire Club</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Sorrow and Plasma drops in total</t>
+          <t>Demonlord drops in total</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
@@ -3339,15 +3421,17 @@
         </is>
       </c>
       <c r="F60" s="4" t="n">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="G60" s="4" t="n">
-        <v>250</v>
+        <v>10</v>
       </c>
       <c r="H60" s="4" t="n">
-        <v>500</v>
-      </c>
-      <c r="I60" s="4" t="n"/>
+        <v>25</v>
+      </c>
+      <c r="I60" s="4" t="n">
+        <v>50</v>
+      </c>
       <c r="J60" s="3" t="inlineStr">
         <is>
           <t>No</t>
@@ -3363,479 +3447,2437 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="M60" s="3" t="n"/>
+      <c r="M60" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
-      <c r="A61" s="3" t="n"/>
-      <c r="B61" s="3" t="n"/>
-      <c r="C61" s="3" t="n"/>
-      <c r="D61" s="3" t="n"/>
-      <c r="E61" s="3" t="n"/>
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>hellion_seventh_circle</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>Hellion</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>Seventh Circle</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>Every Demonlord drop</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
       <c r="F61" s="4" t="n"/>
       <c r="G61" s="4" t="n"/>
       <c r="H61" s="4" t="n"/>
       <c r="I61" s="4" t="n"/>
-      <c r="J61" s="3" t="n"/>
-      <c r="K61" s="2" t="n"/>
-      <c r="L61" s="3" t="n"/>
-      <c r="M61" s="3" t="n"/>
+      <c r="J61" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L61" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M61" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
-      <c r="A62" s="3" t="n"/>
-      <c r="B62" s="3" t="n"/>
-      <c r="C62" s="3" t="n"/>
-      <c r="D62" s="3" t="n"/>
-      <c r="E62" s="3" t="n"/>
-      <c r="F62" s="4" t="n"/>
-      <c r="G62" s="4" t="n"/>
-      <c r="H62" s="4" t="n"/>
-      <c r="I62" s="4" t="n"/>
-      <c r="J62" s="3" t="n"/>
-      <c r="K62" s="2" t="n"/>
-      <c r="L62" s="3" t="n"/>
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>lava_magma_maker</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>Eruption</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>Magma Maker</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>Rare lava creatures killed</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>Tiered</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="G62" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="H62" s="4" t="n">
+        <v>500</v>
+      </c>
+      <c r="I62" s="4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="J62" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L62" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="M62" s="3" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="3" t="n"/>
-      <c r="B63" s="3" t="n"/>
-      <c r="C63" s="3" t="n"/>
-      <c r="D63" s="3" t="n"/>
-      <c r="E63" s="3" t="n"/>
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>lava_flash</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>Eruption</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>In a Flash</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>Flash I</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
       <c r="F63" s="4" t="n"/>
       <c r="G63" s="4" t="n"/>
       <c r="H63" s="4" t="n"/>
       <c r="I63" s="4" t="n"/>
-      <c r="J63" s="3" t="n"/>
-      <c r="K63" s="2" t="n"/>
-      <c r="L63" s="3" t="n"/>
+      <c r="J63" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L63" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="M63" s="3" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="3" t="n"/>
-      <c r="B64" s="3" t="n"/>
-      <c r="C64" s="3" t="n"/>
-      <c r="D64" s="3" t="n"/>
-      <c r="E64" s="3" t="n"/>
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>lava_meltdown</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>Eruption</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>Meltdown</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>Radioactive Vial</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
       <c r="F64" s="4" t="n"/>
       <c r="G64" s="4" t="n"/>
       <c r="H64" s="4" t="n"/>
       <c r="I64" s="4" t="n"/>
-      <c r="J64" s="3" t="n"/>
-      <c r="K64" s="2" t="n"/>
-      <c r="L64" s="3" t="n"/>
+      <c r="J64" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L64" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="M64" s="3" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="3" t="n"/>
-      <c r="B65" s="3" t="n"/>
-      <c r="C65" s="3" t="n"/>
-      <c r="D65" s="3" t="n"/>
-      <c r="E65" s="3" t="n"/>
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>lava_end_times</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>Eruption</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>End Times</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>Burnt Texts</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
       <c r="F65" s="4" t="n"/>
       <c r="G65" s="4" t="n"/>
       <c r="H65" s="4" t="n"/>
       <c r="I65" s="4" t="n"/>
-      <c r="J65" s="3" t="n"/>
-      <c r="K65" s="2" t="n"/>
-      <c r="L65" s="3" t="n"/>
+      <c r="J65" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L65" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="M65" s="3" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="3" t="n"/>
-      <c r="B66" s="3" t="n"/>
-      <c r="C66" s="3" t="n"/>
-      <c r="D66" s="3" t="n"/>
-      <c r="E66" s="3" t="n"/>
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>lava_kuudra</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>Eruption</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>Kuudra Rises</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>Carmine Dye</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
       <c r="F66" s="4" t="n"/>
       <c r="G66" s="4" t="n"/>
       <c r="H66" s="4" t="n"/>
       <c r="I66" s="4" t="n"/>
-      <c r="J66" s="3" t="n"/>
-      <c r="K66" s="2" t="n"/>
-      <c r="L66" s="3" t="n"/>
+      <c r="J66" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L66" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="M66" s="3" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="3" t="n"/>
-      <c r="B67" s="3" t="n"/>
-      <c r="C67" s="3" t="n"/>
-      <c r="D67" s="3" t="n"/>
-      <c r="E67" s="3" t="n"/>
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>lava_jaw_dropping</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>Eruption</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>Jaw Dropping</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>Any win from a Lord Jawbus</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
       <c r="F67" s="4" t="n"/>
       <c r="G67" s="4" t="n"/>
       <c r="H67" s="4" t="n"/>
       <c r="I67" s="4" t="n"/>
-      <c r="J67" s="3" t="n"/>
-      <c r="K67" s="2" t="n"/>
-      <c r="L67" s="3" t="n"/>
+      <c r="J67" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L67" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="M67" s="3" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="3" t="n"/>
-      <c r="B68" s="3" t="n"/>
-      <c r="C68" s="3" t="n"/>
-      <c r="D68" s="3" t="n"/>
-      <c r="E68" s="3" t="n"/>
-      <c r="F68" s="4" t="n"/>
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>lava_thermal_runaway</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>Eruption</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>Thermal Runaway</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>Kills in a row with no win</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="F68" s="4" t="n">
+        <v>50</v>
+      </c>
       <c r="G68" s="4" t="n"/>
       <c r="H68" s="4" t="n"/>
       <c r="I68" s="4" t="n"/>
-      <c r="J68" s="3" t="n"/>
-      <c r="K68" s="2" t="n"/>
-      <c r="L68" s="3" t="n"/>
+      <c r="J68" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>Partly</t>
+        </is>
+      </c>
+      <c r="L68" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="M68" s="3" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="3" t="n"/>
-      <c r="B69" s="3" t="n"/>
-      <c r="C69" s="3" t="n"/>
-      <c r="D69" s="3" t="n"/>
-      <c r="E69" s="3" t="n"/>
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>lava_chained</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>Eruption</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>Chained</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>Chain of the End Times</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
       <c r="F69" s="4" t="n"/>
       <c r="G69" s="4" t="n"/>
       <c r="H69" s="4" t="n"/>
       <c r="I69" s="4" t="n"/>
-      <c r="J69" s="3" t="n"/>
-      <c r="K69" s="2" t="n"/>
-      <c r="L69" s="3" t="n"/>
-      <c r="M69" s="3" t="n"/>
+      <c r="J69" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K69" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L69" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M69" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
-      <c r="A70" s="3" t="n"/>
-      <c r="B70" s="3" t="n"/>
-      <c r="C70" s="3" t="n"/>
-      <c r="D70" s="3" t="n"/>
-      <c r="E70" s="3" t="n"/>
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>lava_pinch_me</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>Eruption</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>Pinch Me</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>Severed Pincer</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
       <c r="F70" s="4" t="n"/>
       <c r="G70" s="4" t="n"/>
       <c r="H70" s="4" t="n"/>
       <c r="I70" s="4" t="n"/>
-      <c r="J70" s="3" t="n"/>
-      <c r="K70" s="2" t="n"/>
-      <c r="L70" s="3" t="n"/>
-      <c r="M70" s="3" t="n"/>
+      <c r="J70" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K70" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L70" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M70" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
-      <c r="A71" s="3" t="n"/>
-      <c r="B71" s="3" t="n"/>
-      <c r="C71" s="3" t="n"/>
-      <c r="D71" s="3" t="n"/>
-      <c r="E71" s="3" t="n"/>
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>lava_forged</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>Eruption</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>Forged in Fire</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>Brimstone Handle</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
       <c r="F71" s="4" t="n"/>
       <c r="G71" s="4" t="n"/>
       <c r="H71" s="4" t="n"/>
       <c r="I71" s="4" t="n"/>
-      <c r="J71" s="3" t="n"/>
-      <c r="K71" s="2" t="n"/>
-      <c r="L71" s="3" t="n"/>
-      <c r="M71" s="3" t="n"/>
+      <c r="J71" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K71" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L71" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M71" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
-      <c r="A72" s="3" t="n"/>
-      <c r="B72" s="3" t="n"/>
-      <c r="C72" s="3" t="n"/>
-      <c r="D72" s="3" t="n"/>
-      <c r="E72" s="3" t="n"/>
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>lava_shell_shocked</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>Eruption</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>Shell Shocked</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>Scuttler Shell</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
       <c r="F72" s="4" t="n"/>
       <c r="G72" s="4" t="n"/>
       <c r="H72" s="4" t="n"/>
       <c r="I72" s="4" t="n"/>
-      <c r="J72" s="3" t="n"/>
-      <c r="K72" s="2" t="n"/>
-      <c r="L72" s="3" t="n"/>
-      <c r="M72" s="3" t="n"/>
+      <c r="J72" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L72" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M72" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
-      <c r="A73" s="3" t="n"/>
-      <c r="B73" s="3" t="n"/>
-      <c r="C73" s="3" t="n"/>
-      <c r="D73" s="3" t="n"/>
-      <c r="E73" s="3" t="n"/>
-      <c r="F73" s="4" t="n"/>
-      <c r="G73" s="4" t="n"/>
-      <c r="H73" s="4" t="n"/>
-      <c r="I73" s="4" t="n"/>
-      <c r="J73" s="3" t="n"/>
-      <c r="K73" s="2" t="n"/>
-      <c r="L73" s="3" t="n"/>
-      <c r="M73" s="3" t="n"/>
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>lava_hot_catch</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>Eruption</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>Hot Catch</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>Lava creature drops in total</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>Tiered</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G73" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="H73" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="I73" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="J73" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K73" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L73" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M73" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
-      <c r="A74" s="3" t="n"/>
-      <c r="B74" s="3" t="n"/>
-      <c r="C74" s="3" t="n"/>
-      <c r="D74" s="3" t="n"/>
-      <c r="E74" s="3" t="n"/>
-      <c r="F74" s="4" t="n"/>
-      <c r="G74" s="4" t="n"/>
-      <c r="H74" s="4" t="n"/>
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>fin_shark_week</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>Fin</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>Shark Week</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>Great White Sharks killed</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>Tiered</t>
+        </is>
+      </c>
+      <c r="F74" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="G74" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="H74" s="4" t="n">
+        <v>500</v>
+      </c>
       <c r="I74" s="4" t="n"/>
-      <c r="J74" s="3" t="n"/>
-      <c r="K74" s="2" t="n"/>
-      <c r="L74" s="3" t="n"/>
+      <c r="J74" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K74" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L74" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="M74" s="3" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="3" t="n"/>
-      <c r="B75" s="3" t="n"/>
-      <c r="C75" s="3" t="n"/>
-      <c r="D75" s="3" t="n"/>
-      <c r="E75" s="3" t="n"/>
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>fin_big_fish</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>Fin</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>Big Fish</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>A Megalodon (any rarity)</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
       <c r="F75" s="4" t="n"/>
       <c r="G75" s="4" t="n"/>
       <c r="H75" s="4" t="n"/>
       <c r="I75" s="4" t="n"/>
-      <c r="J75" s="3" t="n"/>
-      <c r="K75" s="2" t="n"/>
-      <c r="L75" s="3" t="n"/>
-      <c r="M75" s="3" t="n"/>
+      <c r="J75" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K75" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L75" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M75" s="3" t="inlineStr">
+        <is>
+          <t>Claude: was 'Epic Megalodon'. The stats never kept the pet's rarity, so any Megalodon counts; Bigger Fish stays legendary-only, counted from the update.</t>
+        </is>
+      </c>
     </row>
     <row r="76">
-      <c r="A76" s="3" t="n"/>
-      <c r="B76" s="3" t="n"/>
-      <c r="C76" s="3" t="n"/>
-      <c r="D76" s="3" t="n"/>
-      <c r="E76" s="3" t="n"/>
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>fin_bigger_fish</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>Fin</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>Bigger Fish</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>Legendary Megalodon</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
       <c r="F76" s="4" t="n"/>
       <c r="G76" s="4" t="n"/>
       <c r="H76" s="4" t="n"/>
       <c r="I76" s="4" t="n"/>
-      <c r="J76" s="3" t="n"/>
-      <c r="K76" s="2" t="n"/>
-      <c r="L76" s="3" t="n"/>
+      <c r="J76" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K76" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L76" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="M76" s="3" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="3" t="n"/>
-      <c r="B77" s="3" t="n"/>
-      <c r="C77" s="3" t="n"/>
-      <c r="D77" s="3" t="n"/>
-      <c r="E77" s="3" t="n"/>
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>fin_tooth_fairy</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>Fin</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>Tooth Fairy</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>Great White Shark Tooth</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
       <c r="F77" s="4" t="n"/>
       <c r="G77" s="4" t="n"/>
       <c r="H77" s="4" t="n"/>
       <c r="I77" s="4" t="n"/>
-      <c r="J77" s="3" t="n"/>
-      <c r="K77" s="2" t="n"/>
-      <c r="L77" s="3" t="n"/>
+      <c r="J77" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K77" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L77" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="M77" s="3" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="3" t="n"/>
-      <c r="B78" s="3" t="n"/>
-      <c r="C78" s="3" t="n"/>
-      <c r="D78" s="3" t="n"/>
-      <c r="E78" s="3" t="n"/>
-      <c r="F78" s="4" t="n"/>
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>fin_off_the_hook</t>
+        </is>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>Fin</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>Off the Hook</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>Sharks that dropped neither</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="F78" s="4" t="n">
+        <v>50</v>
+      </c>
       <c r="G78" s="4" t="n"/>
       <c r="H78" s="4" t="n"/>
       <c r="I78" s="4" t="n"/>
-      <c r="J78" s="3" t="n"/>
-      <c r="K78" s="2" t="n"/>
-      <c r="L78" s="3" t="n"/>
+      <c r="J78" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K78" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L78" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="M78" s="3" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="3" t="n"/>
-      <c r="B79" s="3" t="n"/>
-      <c r="C79" s="3" t="n"/>
-      <c r="D79" s="3" t="n"/>
-      <c r="E79" s="3" t="n"/>
-      <c r="F79" s="4" t="n"/>
-      <c r="G79" s="4" t="n"/>
-      <c r="H79" s="4" t="n"/>
-      <c r="I79" s="4" t="n"/>
-      <c r="J79" s="3" t="n"/>
-      <c r="K79" s="2" t="n"/>
-      <c r="L79" s="3" t="n"/>
-      <c r="M79" s="3" t="n"/>
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>fin_dentist</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>Fin</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>Dentist</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>Great White Shark Teeth in total</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="inlineStr">
+        <is>
+          <t>Tiered</t>
+        </is>
+      </c>
+      <c r="F79" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G79" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="H79" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="I79" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="J79" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K79" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L79" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M79" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
-      <c r="A80" s="3" t="n"/>
-      <c r="B80" s="3" t="n"/>
-      <c r="C80" s="3" t="n"/>
-      <c r="D80" s="3" t="n"/>
-      <c r="E80" s="3" t="n"/>
-      <c r="F80" s="4" t="n"/>
-      <c r="G80" s="4" t="n"/>
-      <c r="H80" s="4" t="n"/>
-      <c r="I80" s="4" t="n"/>
-      <c r="J80" s="3" t="n"/>
-      <c r="K80" s="2" t="n"/>
-      <c r="L80" s="3" t="n"/>
-      <c r="M80" s="3" t="n"/>
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>fin_school</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>Fin</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>School is In</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>Megalodons in total</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="inlineStr">
+        <is>
+          <t>Tiered</t>
+        </is>
+      </c>
+      <c r="F80" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G80" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="H80" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I80" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="J80" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K80" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L80" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M80" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
-      <c r="A81" s="3" t="n"/>
-      <c r="B81" s="3" t="n"/>
-      <c r="C81" s="3" t="n"/>
-      <c r="D81" s="3" t="n"/>
-      <c r="E81" s="3" t="n"/>
-      <c r="F81" s="4" t="n"/>
-      <c r="G81" s="4" t="n"/>
-      <c r="H81" s="4" t="n"/>
-      <c r="I81" s="4" t="n"/>
-      <c r="J81" s="3" t="n"/>
-      <c r="K81" s="2" t="n"/>
-      <c r="L81" s="3" t="n"/>
-      <c r="M81" s="3" t="n"/>
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>fin_dry_dock</t>
+        </is>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>Fin</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>Dry Dock</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>Sharks in a row with no drop</t>
+        </is>
+      </c>
+      <c r="E81" s="3" t="inlineStr">
+        <is>
+          <t>Tiered</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="G81" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="H81" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="I81" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="J81" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K81" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L81" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M81" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+        </is>
+      </c>
     </row>
     <row r="82">
-      <c r="A82" s="3" t="n"/>
-      <c r="B82" s="3" t="n"/>
-      <c r="C82" s="3" t="n"/>
-      <c r="D82" s="3" t="n"/>
-      <c r="E82" s="3" t="n"/>
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>fin_feeding_frenzy</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>Fin</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>Feeding Frenzy</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>Two shark drops within 10 minutes</t>
+        </is>
+      </c>
+      <c r="E82" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
       <c r="F82" s="4" t="n"/>
       <c r="G82" s="4" t="n"/>
       <c r="H82" s="4" t="n"/>
       <c r="I82" s="4" t="n"/>
-      <c r="J82" s="3" t="n"/>
-      <c r="K82" s="2" t="n"/>
-      <c r="L82" s="3" t="n"/>
-      <c r="M82" s="3" t="n"/>
+      <c r="J82" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K82" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L82" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M82" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+        </is>
+      </c>
     </row>
     <row r="83">
-      <c r="A83" s="3" t="n"/>
-      <c r="B83" s="3" t="n"/>
-      <c r="C83" s="3" t="n"/>
-      <c r="D83" s="3" t="n"/>
-      <c r="E83" s="3" t="n"/>
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>fin_both_ends</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>Fin</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>Both Ends</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>A Megalodon and a Tooth</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
       <c r="F83" s="4" t="n"/>
       <c r="G83" s="4" t="n"/>
       <c r="H83" s="4" t="n"/>
       <c r="I83" s="4" t="n"/>
-      <c r="J83" s="3" t="n"/>
-      <c r="K83" s="2" t="n"/>
-      <c r="L83" s="3" t="n"/>
-      <c r="M83" s="3" t="n"/>
+      <c r="J83" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K83" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L83" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M83" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+        </is>
+      </c>
     </row>
     <row r="84">
-      <c r="A84" s="3" t="n"/>
-      <c r="B84" s="3" t="n"/>
-      <c r="C84" s="3" t="n"/>
-      <c r="D84" s="3" t="n"/>
-      <c r="E84" s="3" t="n"/>
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>wisp_sorrowful</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>Wisp</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>Sorrowful</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>Sorrow</t>
+        </is>
+      </c>
+      <c r="E84" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
       <c r="F84" s="4" t="n"/>
       <c r="G84" s="4" t="n"/>
       <c r="H84" s="4" t="n"/>
       <c r="I84" s="4" t="n"/>
-      <c r="J84" s="3" t="n"/>
-      <c r="K84" s="2" t="n"/>
-      <c r="L84" s="3" t="n"/>
+      <c r="J84" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K84" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L84" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="M84" s="3" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="3" t="n"/>
-      <c r="B85" s="3" t="n"/>
-      <c r="C85" s="3" t="n"/>
-      <c r="D85" s="3" t="n"/>
-      <c r="E85" s="3" t="n"/>
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>wisp_plasma</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>Wisp</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>Plasma Screen</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>Plasma</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
       <c r="F85" s="4" t="n"/>
       <c r="G85" s="4" t="n"/>
       <c r="H85" s="4" t="n"/>
       <c r="I85" s="4" t="n"/>
-      <c r="J85" s="3" t="n"/>
-      <c r="K85" s="2" t="n"/>
-      <c r="L85" s="3" t="n"/>
+      <c r="J85" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K85" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L85" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="M85" s="3" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="3" t="n"/>
-      <c r="B86" s="3" t="n"/>
-      <c r="C86" s="3" t="n"/>
-      <c r="D86" s="3" t="n"/>
-      <c r="E86" s="3" t="n"/>
-      <c r="F86" s="4" t="n"/>
-      <c r="G86" s="4" t="n"/>
-      <c r="H86" s="4" t="n"/>
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>wisp_spirit_level</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>Wisp</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>Spirit Level</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>Sorrow and Plasma drops in total</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="inlineStr">
+        <is>
+          <t>Tiered</t>
+        </is>
+      </c>
+      <c r="F86" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="G86" s="4" t="n">
+        <v>250</v>
+      </c>
+      <c r="H86" s="4" t="n">
+        <v>500</v>
+      </c>
       <c r="I86" s="4" t="n"/>
-      <c r="J86" s="3" t="n"/>
-      <c r="K86" s="2" t="n"/>
-      <c r="L86" s="3" t="n"/>
+      <c r="J86" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K86" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L86" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="M86" s="3" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" s="3" t="n"/>
-      <c r="B87" s="3" t="n"/>
-      <c r="C87" s="3" t="n"/>
-      <c r="D87" s="3" t="n"/>
-      <c r="E87" s="3" t="n"/>
-      <c r="F87" s="4" t="n"/>
-      <c r="G87" s="4" t="n"/>
-      <c r="H87" s="4" t="n"/>
-      <c r="I87" s="4" t="n"/>
-      <c r="J87" s="3" t="n"/>
-      <c r="K87" s="2" t="n"/>
-      <c r="L87" s="3" t="n"/>
-      <c r="M87" s="3" t="n"/>
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>wisp_drowning</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>Wisp</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>Drowning in Sorrow</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>Sorrow drops in total</t>
+        </is>
+      </c>
+      <c r="E87" s="3" t="inlineStr">
+        <is>
+          <t>Tiered</t>
+        </is>
+      </c>
+      <c r="F87" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G87" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="H87" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="I87" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="J87" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K87" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L87" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M87" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+        </is>
+      </c>
     </row>
     <row r="88">
-      <c r="A88" s="3" t="n"/>
-      <c r="B88" s="3" t="n"/>
-      <c r="C88" s="3" t="n"/>
-      <c r="D88" s="3" t="n"/>
-      <c r="E88" s="3" t="n"/>
-      <c r="F88" s="4" t="n"/>
-      <c r="G88" s="4" t="n"/>
-      <c r="H88" s="4" t="n"/>
-      <c r="I88" s="4" t="n"/>
-      <c r="J88" s="3" t="n"/>
-      <c r="K88" s="2" t="n"/>
-      <c r="L88" s="3" t="n"/>
-      <c r="M88" s="3" t="n"/>
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>wisp_high_voltage</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>Wisp</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>High Voltage</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>Plasma drops in total</t>
+        </is>
+      </c>
+      <c r="E88" s="3" t="inlineStr">
+        <is>
+          <t>Tiered</t>
+        </is>
+      </c>
+      <c r="F88" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G88" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="H88" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="I88" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="J88" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K88" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L88" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M88" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+        </is>
+      </c>
     </row>
     <row r="89">
-      <c r="A89" s="3" t="n"/>
-      <c r="B89" s="3" t="n"/>
-      <c r="C89" s="3" t="n"/>
-      <c r="D89" s="3" t="n"/>
-      <c r="E89" s="3" t="n"/>
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>wisp_bittersweet</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>Wisp</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>Bittersweet</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>Both Sorrow and Plasma</t>
+        </is>
+      </c>
+      <c r="E89" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
       <c r="F89" s="4" t="n"/>
       <c r="G89" s="4" t="n"/>
       <c r="H89" s="4" t="n"/>
       <c r="I89" s="4" t="n"/>
-      <c r="J89" s="3" t="n"/>
-      <c r="K89" s="2" t="n"/>
-      <c r="L89" s="3" t="n"/>
-      <c r="M89" s="3" t="n"/>
+      <c r="J89" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K89" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L89" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M89" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+        </is>
+      </c>
     </row>
     <row r="90">
-      <c r="A90" s="3" t="n"/>
-      <c r="B90" s="3" t="n"/>
-      <c r="C90" s="3" t="n"/>
-      <c r="D90" s="3" t="n"/>
-      <c r="E90" s="3" t="n"/>
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>wisp_double_haunting</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>Wisp</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>Double Haunting</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>Two Ghost drops within 10 minutes</t>
+        </is>
+      </c>
+      <c r="E90" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
       <c r="F90" s="4" t="n"/>
       <c r="G90" s="4" t="n"/>
       <c r="H90" s="4" t="n"/>
       <c r="I90" s="4" t="n"/>
-      <c r="J90" s="3" t="n"/>
-      <c r="K90" s="2" t="n"/>
-      <c r="L90" s="3" t="n"/>
-      <c r="M90" s="3" t="n"/>
+      <c r="J90" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K90" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L90" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M90" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>wisp_poltergeist</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>Wisp</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>Poltergeist</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>Three Ghost drops within an hour</t>
+        </is>
+      </c>
+      <c r="E91" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="F91" s="4" t="n"/>
+      <c r="G91" s="4" t="n"/>
+      <c r="H91" s="4" t="n"/>
+      <c r="I91" s="4" t="n"/>
+      <c r="J91" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K91" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L91" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M91" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>wisp_matched_pair</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>Wisp</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>Matched Pair</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>Sorrow and Plasma within an hour of each other</t>
+        </is>
+      </c>
+      <c r="E92" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="F92" s="4" t="n"/>
+      <c r="G92" s="4" t="n"/>
+      <c r="H92" s="4" t="n"/>
+      <c r="I92" s="4" t="n"/>
+      <c r="J92" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K92" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L92" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M92" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>wisp_witching_hour</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>Wisp</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>Witching Hour</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>A Ghost drop between midnight and 1 AM</t>
+        </is>
+      </c>
+      <c r="E93" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="F93" s="4" t="n"/>
+      <c r="G93" s="4" t="n"/>
+      <c r="H93" s="4" t="n"/>
+      <c r="I93" s="4" t="n"/>
+      <c r="J93" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K93" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L93" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M93" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n"/>
+      <c r="B94" s="3" t="n"/>
+      <c r="C94" s="3" t="n"/>
+      <c r="D94" s="3" t="n"/>
+      <c r="E94" s="3" t="n"/>
+      <c r="F94" s="4" t="n"/>
+      <c r="G94" s="4" t="n"/>
+      <c r="H94" s="4" t="n"/>
+      <c r="I94" s="4" t="n"/>
+      <c r="J94" s="3" t="n"/>
+      <c r="K94" s="2" t="n"/>
+      <c r="L94" s="3" t="n"/>
+      <c r="M94" s="3" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n"/>
+      <c r="B95" s="3" t="n"/>
+      <c r="C95" s="3" t="n"/>
+      <c r="D95" s="3" t="n"/>
+      <c r="E95" s="3" t="n"/>
+      <c r="F95" s="4" t="n"/>
+      <c r="G95" s="4" t="n"/>
+      <c r="H95" s="4" t="n"/>
+      <c r="I95" s="4" t="n"/>
+      <c r="J95" s="3" t="n"/>
+      <c r="K95" s="2" t="n"/>
+      <c r="L95" s="3" t="n"/>
+      <c r="M95" s="3" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n"/>
+      <c r="B96" s="3" t="n"/>
+      <c r="C96" s="3" t="n"/>
+      <c r="D96" s="3" t="n"/>
+      <c r="E96" s="3" t="n"/>
+      <c r="F96" s="4" t="n"/>
+      <c r="G96" s="4" t="n"/>
+      <c r="H96" s="4" t="n"/>
+      <c r="I96" s="4" t="n"/>
+      <c r="J96" s="3" t="n"/>
+      <c r="K96" s="2" t="n"/>
+      <c r="L96" s="3" t="n"/>
+      <c r="M96" s="3" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n"/>
+      <c r="B97" s="3" t="n"/>
+      <c r="C97" s="3" t="n"/>
+      <c r="D97" s="3" t="n"/>
+      <c r="E97" s="3" t="n"/>
+      <c r="F97" s="4" t="n"/>
+      <c r="G97" s="4" t="n"/>
+      <c r="H97" s="4" t="n"/>
+      <c r="I97" s="4" t="n"/>
+      <c r="J97" s="3" t="n"/>
+      <c r="K97" s="2" t="n"/>
+      <c r="L97" s="3" t="n"/>
+      <c r="M97" s="3" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="n"/>
+      <c r="B98" s="3" t="n"/>
+      <c r="C98" s="3" t="n"/>
+      <c r="D98" s="3" t="n"/>
+      <c r="E98" s="3" t="n"/>
+      <c r="F98" s="4" t="n"/>
+      <c r="G98" s="4" t="n"/>
+      <c r="H98" s="4" t="n"/>
+      <c r="I98" s="4" t="n"/>
+      <c r="J98" s="3" t="n"/>
+      <c r="K98" s="2" t="n"/>
+      <c r="L98" s="3" t="n"/>
+      <c r="M98" s="3" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="n"/>
+      <c r="B99" s="3" t="n"/>
+      <c r="C99" s="3" t="n"/>
+      <c r="D99" s="3" t="n"/>
+      <c r="E99" s="3" t="n"/>
+      <c r="F99" s="4" t="n"/>
+      <c r="G99" s="4" t="n"/>
+      <c r="H99" s="4" t="n"/>
+      <c r="I99" s="4" t="n"/>
+      <c r="J99" s="3" t="n"/>
+      <c r="K99" s="2" t="n"/>
+      <c r="L99" s="3" t="n"/>
+      <c r="M99" s="3" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="n"/>
+      <c r="B100" s="3" t="n"/>
+      <c r="C100" s="3" t="n"/>
+      <c r="D100" s="3" t="n"/>
+      <c r="E100" s="3" t="n"/>
+      <c r="F100" s="4" t="n"/>
+      <c r="G100" s="4" t="n"/>
+      <c r="H100" s="4" t="n"/>
+      <c r="I100" s="4" t="n"/>
+      <c r="J100" s="3" t="n"/>
+      <c r="K100" s="2" t="n"/>
+      <c r="L100" s="3" t="n"/>
+      <c r="M100" s="3" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="n"/>
+      <c r="B101" s="3" t="n"/>
+      <c r="C101" s="3" t="n"/>
+      <c r="D101" s="3" t="n"/>
+      <c r="E101" s="3" t="n"/>
+      <c r="F101" s="4" t="n"/>
+      <c r="G101" s="4" t="n"/>
+      <c r="H101" s="4" t="n"/>
+      <c r="I101" s="4" t="n"/>
+      <c r="J101" s="3" t="n"/>
+      <c r="K101" s="2" t="n"/>
+      <c r="L101" s="3" t="n"/>
+      <c r="M101" s="3" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="n"/>
+      <c r="B102" s="3" t="n"/>
+      <c r="C102" s="3" t="n"/>
+      <c r="D102" s="3" t="n"/>
+      <c r="E102" s="3" t="n"/>
+      <c r="F102" s="4" t="n"/>
+      <c r="G102" s="4" t="n"/>
+      <c r="H102" s="4" t="n"/>
+      <c r="I102" s="4" t="n"/>
+      <c r="J102" s="3" t="n"/>
+      <c r="K102" s="2" t="n"/>
+      <c r="L102" s="3" t="n"/>
+      <c r="M102" s="3" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="n"/>
+      <c r="B103" s="3" t="n"/>
+      <c r="C103" s="3" t="n"/>
+      <c r="D103" s="3" t="n"/>
+      <c r="E103" s="3" t="n"/>
+      <c r="F103" s="4" t="n"/>
+      <c r="G103" s="4" t="n"/>
+      <c r="H103" s="4" t="n"/>
+      <c r="I103" s="4" t="n"/>
+      <c r="J103" s="3" t="n"/>
+      <c r="K103" s="2" t="n"/>
+      <c r="L103" s="3" t="n"/>
+      <c r="M103" s="3" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="n"/>
+      <c r="B104" s="3" t="n"/>
+      <c r="C104" s="3" t="n"/>
+      <c r="D104" s="3" t="n"/>
+      <c r="E104" s="3" t="n"/>
+      <c r="F104" s="4" t="n"/>
+      <c r="G104" s="4" t="n"/>
+      <c r="H104" s="4" t="n"/>
+      <c r="I104" s="4" t="n"/>
+      <c r="J104" s="3" t="n"/>
+      <c r="K104" s="2" t="n"/>
+      <c r="L104" s="3" t="n"/>
+      <c r="M104" s="3" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="n"/>
+      <c r="B105" s="3" t="n"/>
+      <c r="C105" s="3" t="n"/>
+      <c r="D105" s="3" t="n"/>
+      <c r="E105" s="3" t="n"/>
+      <c r="F105" s="4" t="n"/>
+      <c r="G105" s="4" t="n"/>
+      <c r="H105" s="4" t="n"/>
+      <c r="I105" s="4" t="n"/>
+      <c r="J105" s="3" t="n"/>
+      <c r="K105" s="2" t="n"/>
+      <c r="L105" s="3" t="n"/>
+      <c r="M105" s="3" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="n"/>
+      <c r="B106" s="3" t="n"/>
+      <c r="C106" s="3" t="n"/>
+      <c r="D106" s="3" t="n"/>
+      <c r="E106" s="3" t="n"/>
+      <c r="F106" s="4" t="n"/>
+      <c r="G106" s="4" t="n"/>
+      <c r="H106" s="4" t="n"/>
+      <c r="I106" s="4" t="n"/>
+      <c r="J106" s="3" t="n"/>
+      <c r="K106" s="2" t="n"/>
+      <c r="L106" s="3" t="n"/>
+      <c r="M106" s="3" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="n"/>
+      <c r="B107" s="3" t="n"/>
+      <c r="C107" s="3" t="n"/>
+      <c r="D107" s="3" t="n"/>
+      <c r="E107" s="3" t="n"/>
+      <c r="F107" s="4" t="n"/>
+      <c r="G107" s="4" t="n"/>
+      <c r="H107" s="4" t="n"/>
+      <c r="I107" s="4" t="n"/>
+      <c r="J107" s="3" t="n"/>
+      <c r="K107" s="2" t="n"/>
+      <c r="L107" s="3" t="n"/>
+      <c r="M107" s="3" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="n"/>
+      <c r="B108" s="3" t="n"/>
+      <c r="C108" s="3" t="n"/>
+      <c r="D108" s="3" t="n"/>
+      <c r="E108" s="3" t="n"/>
+      <c r="F108" s="4" t="n"/>
+      <c r="G108" s="4" t="n"/>
+      <c r="H108" s="4" t="n"/>
+      <c r="I108" s="4" t="n"/>
+      <c r="J108" s="3" t="n"/>
+      <c r="K108" s="2" t="n"/>
+      <c r="L108" s="3" t="n"/>
+      <c r="M108" s="3" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="n"/>
+      <c r="B109" s="3" t="n"/>
+      <c r="C109" s="3" t="n"/>
+      <c r="D109" s="3" t="n"/>
+      <c r="E109" s="3" t="n"/>
+      <c r="F109" s="4" t="n"/>
+      <c r="G109" s="4" t="n"/>
+      <c r="H109" s="4" t="n"/>
+      <c r="I109" s="4" t="n"/>
+      <c r="J109" s="3" t="n"/>
+      <c r="K109" s="2" t="n"/>
+      <c r="L109" s="3" t="n"/>
+      <c r="M109" s="3" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="n"/>
+      <c r="B110" s="3" t="n"/>
+      <c r="C110" s="3" t="n"/>
+      <c r="D110" s="3" t="n"/>
+      <c r="E110" s="3" t="n"/>
+      <c r="F110" s="4" t="n"/>
+      <c r="G110" s="4" t="n"/>
+      <c r="H110" s="4" t="n"/>
+      <c r="I110" s="4" t="n"/>
+      <c r="J110" s="3" t="n"/>
+      <c r="K110" s="2" t="n"/>
+      <c r="L110" s="3" t="n"/>
+      <c r="M110" s="3" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="n"/>
+      <c r="B111" s="3" t="n"/>
+      <c r="C111" s="3" t="n"/>
+      <c r="D111" s="3" t="n"/>
+      <c r="E111" s="3" t="n"/>
+      <c r="F111" s="4" t="n"/>
+      <c r="G111" s="4" t="n"/>
+      <c r="H111" s="4" t="n"/>
+      <c r="I111" s="4" t="n"/>
+      <c r="J111" s="3" t="n"/>
+      <c r="K111" s="2" t="n"/>
+      <c r="L111" s="3" t="n"/>
+      <c r="M111" s="3" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="n"/>
+      <c r="B112" s="3" t="n"/>
+      <c r="C112" s="3" t="n"/>
+      <c r="D112" s="3" t="n"/>
+      <c r="E112" s="3" t="n"/>
+      <c r="F112" s="4" t="n"/>
+      <c r="G112" s="4" t="n"/>
+      <c r="H112" s="4" t="n"/>
+      <c r="I112" s="4" t="n"/>
+      <c r="J112" s="3" t="n"/>
+      <c r="K112" s="2" t="n"/>
+      <c r="L112" s="3" t="n"/>
+      <c r="M112" s="3" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="n"/>
+      <c r="B113" s="3" t="n"/>
+      <c r="C113" s="3" t="n"/>
+      <c r="D113" s="3" t="n"/>
+      <c r="E113" s="3" t="n"/>
+      <c r="F113" s="4" t="n"/>
+      <c r="G113" s="4" t="n"/>
+      <c r="H113" s="4" t="n"/>
+      <c r="I113" s="4" t="n"/>
+      <c r="J113" s="3" t="n"/>
+      <c r="K113" s="2" t="n"/>
+      <c r="L113" s="3" t="n"/>
+      <c r="M113" s="3" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="n"/>
+      <c r="B114" s="3" t="n"/>
+      <c r="C114" s="3" t="n"/>
+      <c r="D114" s="3" t="n"/>
+      <c r="E114" s="3" t="n"/>
+      <c r="F114" s="4" t="n"/>
+      <c r="G114" s="4" t="n"/>
+      <c r="H114" s="4" t="n"/>
+      <c r="I114" s="4" t="n"/>
+      <c r="J114" s="3" t="n"/>
+      <c r="K114" s="2" t="n"/>
+      <c r="L114" s="3" t="n"/>
+      <c r="M114" s="3" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="n"/>
+      <c r="B115" s="3" t="n"/>
+      <c r="C115" s="3" t="n"/>
+      <c r="D115" s="3" t="n"/>
+      <c r="E115" s="3" t="n"/>
+      <c r="F115" s="4" t="n"/>
+      <c r="G115" s="4" t="n"/>
+      <c r="H115" s="4" t="n"/>
+      <c r="I115" s="4" t="n"/>
+      <c r="J115" s="3" t="n"/>
+      <c r="K115" s="2" t="n"/>
+      <c r="L115" s="3" t="n"/>
+      <c r="M115" s="3" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="n"/>
+      <c r="B116" s="3" t="n"/>
+      <c r="C116" s="3" t="n"/>
+      <c r="D116" s="3" t="n"/>
+      <c r="E116" s="3" t="n"/>
+      <c r="F116" s="4" t="n"/>
+      <c r="G116" s="4" t="n"/>
+      <c r="H116" s="4" t="n"/>
+      <c r="I116" s="4" t="n"/>
+      <c r="J116" s="3" t="n"/>
+      <c r="K116" s="2" t="n"/>
+      <c r="L116" s="3" t="n"/>
+      <c r="M116" s="3" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="n"/>
+      <c r="B117" s="3" t="n"/>
+      <c r="C117" s="3" t="n"/>
+      <c r="D117" s="3" t="n"/>
+      <c r="E117" s="3" t="n"/>
+      <c r="F117" s="4" t="n"/>
+      <c r="G117" s="4" t="n"/>
+      <c r="H117" s="4" t="n"/>
+      <c r="I117" s="4" t="n"/>
+      <c r="J117" s="3" t="n"/>
+      <c r="K117" s="2" t="n"/>
+      <c r="L117" s="3" t="n"/>
+      <c r="M117" s="3" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="n"/>
+      <c r="B118" s="3" t="n"/>
+      <c r="C118" s="3" t="n"/>
+      <c r="D118" s="3" t="n"/>
+      <c r="E118" s="3" t="n"/>
+      <c r="F118" s="4" t="n"/>
+      <c r="G118" s="4" t="n"/>
+      <c r="H118" s="4" t="n"/>
+      <c r="I118" s="4" t="n"/>
+      <c r="J118" s="3" t="n"/>
+      <c r="K118" s="2" t="n"/>
+      <c r="L118" s="3" t="n"/>
+      <c r="M118" s="3" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="n"/>
+      <c r="B119" s="3" t="n"/>
+      <c r="C119" s="3" t="n"/>
+      <c r="D119" s="3" t="n"/>
+      <c r="E119" s="3" t="n"/>
+      <c r="F119" s="4" t="n"/>
+      <c r="G119" s="4" t="n"/>
+      <c r="H119" s="4" t="n"/>
+      <c r="I119" s="4" t="n"/>
+      <c r="J119" s="3" t="n"/>
+      <c r="K119" s="2" t="n"/>
+      <c r="L119" s="3" t="n"/>
+      <c r="M119" s="3" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="n"/>
+      <c r="B120" s="3" t="n"/>
+      <c r="C120" s="3" t="n"/>
+      <c r="D120" s="3" t="n"/>
+      <c r="E120" s="3" t="n"/>
+      <c r="F120" s="4" t="n"/>
+      <c r="G120" s="4" t="n"/>
+      <c r="H120" s="4" t="n"/>
+      <c r="I120" s="4" t="n"/>
+      <c r="J120" s="3" t="n"/>
+      <c r="K120" s="2" t="n"/>
+      <c r="L120" s="3" t="n"/>
+      <c r="M120" s="3" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="n"/>
+      <c r="B121" s="3" t="n"/>
+      <c r="C121" s="3" t="n"/>
+      <c r="D121" s="3" t="n"/>
+      <c r="E121" s="3" t="n"/>
+      <c r="F121" s="4" t="n"/>
+      <c r="G121" s="4" t="n"/>
+      <c r="H121" s="4" t="n"/>
+      <c r="I121" s="4" t="n"/>
+      <c r="J121" s="3" t="n"/>
+      <c r="K121" s="2" t="n"/>
+      <c r="L121" s="3" t="n"/>
+      <c r="M121" s="3" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="n"/>
+      <c r="B122" s="3" t="n"/>
+      <c r="C122" s="3" t="n"/>
+      <c r="D122" s="3" t="n"/>
+      <c r="E122" s="3" t="n"/>
+      <c r="F122" s="4" t="n"/>
+      <c r="G122" s="4" t="n"/>
+      <c r="H122" s="4" t="n"/>
+      <c r="I122" s="4" t="n"/>
+      <c r="J122" s="3" t="n"/>
+      <c r="K122" s="2" t="n"/>
+      <c r="L122" s="3" t="n"/>
+      <c r="M122" s="3" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="n"/>
+      <c r="B123" s="3" t="n"/>
+      <c r="C123" s="3" t="n"/>
+      <c r="D123" s="3" t="n"/>
+      <c r="E123" s="3" t="n"/>
+      <c r="F123" s="4" t="n"/>
+      <c r="G123" s="4" t="n"/>
+      <c r="H123" s="4" t="n"/>
+      <c r="I123" s="4" t="n"/>
+      <c r="J123" s="3" t="n"/>
+      <c r="K123" s="2" t="n"/>
+      <c r="L123" s="3" t="n"/>
+      <c r="M123" s="3" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="n"/>
+      <c r="B124" s="3" t="n"/>
+      <c r="C124" s="3" t="n"/>
+      <c r="D124" s="3" t="n"/>
+      <c r="E124" s="3" t="n"/>
+      <c r="F124" s="4" t="n"/>
+      <c r="G124" s="4" t="n"/>
+      <c r="H124" s="4" t="n"/>
+      <c r="I124" s="4" t="n"/>
+      <c r="J124" s="3" t="n"/>
+      <c r="K124" s="2" t="n"/>
+      <c r="L124" s="3" t="n"/>
+      <c r="M124" s="3" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="n"/>
+      <c r="B125" s="3" t="n"/>
+      <c r="C125" s="3" t="n"/>
+      <c r="D125" s="3" t="n"/>
+      <c r="E125" s="3" t="n"/>
+      <c r="F125" s="4" t="n"/>
+      <c r="G125" s="4" t="n"/>
+      <c r="H125" s="4" t="n"/>
+      <c r="I125" s="4" t="n"/>
+      <c r="J125" s="3" t="n"/>
+      <c r="K125" s="2" t="n"/>
+      <c r="L125" s="3" t="n"/>
+      <c r="M125" s="3" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="n"/>
+      <c r="B126" s="3" t="n"/>
+      <c r="C126" s="3" t="n"/>
+      <c r="D126" s="3" t="n"/>
+      <c r="E126" s="3" t="n"/>
+      <c r="F126" s="4" t="n"/>
+      <c r="G126" s="4" t="n"/>
+      <c r="H126" s="4" t="n"/>
+      <c r="I126" s="4" t="n"/>
+      <c r="J126" s="3" t="n"/>
+      <c r="K126" s="2" t="n"/>
+      <c r="L126" s="3" t="n"/>
+      <c r="M126" s="3" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="n"/>
+      <c r="B127" s="3" t="n"/>
+      <c r="C127" s="3" t="n"/>
+      <c r="D127" s="3" t="n"/>
+      <c r="E127" s="3" t="n"/>
+      <c r="F127" s="4" t="n"/>
+      <c r="G127" s="4" t="n"/>
+      <c r="H127" s="4" t="n"/>
+      <c r="I127" s="4" t="n"/>
+      <c r="J127" s="3" t="n"/>
+      <c r="K127" s="2" t="n"/>
+      <c r="L127" s="3" t="n"/>
+      <c r="M127" s="3" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="n"/>
+      <c r="B128" s="3" t="n"/>
+      <c r="C128" s="3" t="n"/>
+      <c r="D128" s="3" t="n"/>
+      <c r="E128" s="3" t="n"/>
+      <c r="F128" s="4" t="n"/>
+      <c r="G128" s="4" t="n"/>
+      <c r="H128" s="4" t="n"/>
+      <c r="I128" s="4" t="n"/>
+      <c r="J128" s="3" t="n"/>
+      <c r="K128" s="2" t="n"/>
+      <c r="L128" s="3" t="n"/>
+      <c r="M128" s="3" t="n"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="n"/>
+      <c r="B129" s="3" t="n"/>
+      <c r="C129" s="3" t="n"/>
+      <c r="D129" s="3" t="n"/>
+      <c r="E129" s="3" t="n"/>
+      <c r="F129" s="4" t="n"/>
+      <c r="G129" s="4" t="n"/>
+      <c r="H129" s="4" t="n"/>
+      <c r="I129" s="4" t="n"/>
+      <c r="J129" s="3" t="n"/>
+      <c r="K129" s="2" t="n"/>
+      <c r="L129" s="3" t="n"/>
+      <c r="M129" s="3" t="n"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="n"/>
+      <c r="B130" s="3" t="n"/>
+      <c r="C130" s="3" t="n"/>
+      <c r="D130" s="3" t="n"/>
+      <c r="E130" s="3" t="n"/>
+      <c r="F130" s="4" t="n"/>
+      <c r="G130" s="4" t="n"/>
+      <c r="H130" s="4" t="n"/>
+      <c r="I130" s="4" t="n"/>
+      <c r="J130" s="3" t="n"/>
+      <c r="K130" s="2" t="n"/>
+      <c r="L130" s="3" t="n"/>
+      <c r="M130" s="3" t="n"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="n"/>
+      <c r="B131" s="3" t="n"/>
+      <c r="C131" s="3" t="n"/>
+      <c r="D131" s="3" t="n"/>
+      <c r="E131" s="3" t="n"/>
+      <c r="F131" s="4" t="n"/>
+      <c r="G131" s="4" t="n"/>
+      <c r="H131" s="4" t="n"/>
+      <c r="I131" s="4" t="n"/>
+      <c r="J131" s="3" t="n"/>
+      <c r="K131" s="2" t="n"/>
+      <c r="L131" s="3" t="n"/>
+      <c r="M131" s="3" t="n"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="n"/>
+      <c r="B132" s="3" t="n"/>
+      <c r="C132" s="3" t="n"/>
+      <c r="D132" s="3" t="n"/>
+      <c r="E132" s="3" t="n"/>
+      <c r="F132" s="4" t="n"/>
+      <c r="G132" s="4" t="n"/>
+      <c r="H132" s="4" t="n"/>
+      <c r="I132" s="4" t="n"/>
+      <c r="J132" s="3" t="n"/>
+      <c r="K132" s="2" t="n"/>
+      <c r="L132" s="3" t="n"/>
+      <c r="M132" s="3" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="n"/>
+      <c r="B133" s="3" t="n"/>
+      <c r="C133" s="3" t="n"/>
+      <c r="D133" s="3" t="n"/>
+      <c r="E133" s="3" t="n"/>
+      <c r="F133" s="4" t="n"/>
+      <c r="G133" s="4" t="n"/>
+      <c r="H133" s="4" t="n"/>
+      <c r="I133" s="4" t="n"/>
+      <c r="J133" s="3" t="n"/>
+      <c r="K133" s="2" t="n"/>
+      <c r="L133" s="3" t="n"/>
+      <c r="M133" s="3" t="n"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="n"/>
+      <c r="B134" s="3" t="n"/>
+      <c r="C134" s="3" t="n"/>
+      <c r="D134" s="3" t="n"/>
+      <c r="E134" s="3" t="n"/>
+      <c r="F134" s="4" t="n"/>
+      <c r="G134" s="4" t="n"/>
+      <c r="H134" s="4" t="n"/>
+      <c r="I134" s="4" t="n"/>
+      <c r="J134" s="3" t="n"/>
+      <c r="K134" s="2" t="n"/>
+      <c r="L134" s="3" t="n"/>
+      <c r="M134" s="3" t="n"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="n"/>
+      <c r="B135" s="3" t="n"/>
+      <c r="C135" s="3" t="n"/>
+      <c r="D135" s="3" t="n"/>
+      <c r="E135" s="3" t="n"/>
+      <c r="F135" s="4" t="n"/>
+      <c r="G135" s="4" t="n"/>
+      <c r="H135" s="4" t="n"/>
+      <c r="I135" s="4" t="n"/>
+      <c r="J135" s="3" t="n"/>
+      <c r="K135" s="2" t="n"/>
+      <c r="L135" s="3" t="n"/>
+      <c r="M135" s="3" t="n"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="n"/>
+      <c r="B136" s="3" t="n"/>
+      <c r="C136" s="3" t="n"/>
+      <c r="D136" s="3" t="n"/>
+      <c r="E136" s="3" t="n"/>
+      <c r="F136" s="4" t="n"/>
+      <c r="G136" s="4" t="n"/>
+      <c r="H136" s="4" t="n"/>
+      <c r="I136" s="4" t="n"/>
+      <c r="J136" s="3" t="n"/>
+      <c r="K136" s="2" t="n"/>
+      <c r="L136" s="3" t="n"/>
+      <c r="M136" s="3" t="n"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="n"/>
+      <c r="B137" s="3" t="n"/>
+      <c r="C137" s="3" t="n"/>
+      <c r="D137" s="3" t="n"/>
+      <c r="E137" s="3" t="n"/>
+      <c r="F137" s="4" t="n"/>
+      <c r="G137" s="4" t="n"/>
+      <c r="H137" s="4" t="n"/>
+      <c r="I137" s="4" t="n"/>
+      <c r="J137" s="3" t="n"/>
+      <c r="K137" s="2" t="n"/>
+      <c r="L137" s="3" t="n"/>
+      <c r="M137" s="3" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="n"/>
+      <c r="B138" s="3" t="n"/>
+      <c r="C138" s="3" t="n"/>
+      <c r="D138" s="3" t="n"/>
+      <c r="E138" s="3" t="n"/>
+      <c r="F138" s="4" t="n"/>
+      <c r="G138" s="4" t="n"/>
+      <c r="H138" s="4" t="n"/>
+      <c r="I138" s="4" t="n"/>
+      <c r="J138" s="3" t="n"/>
+      <c r="K138" s="2" t="n"/>
+      <c r="L138" s="3" t="n"/>
+      <c r="M138" s="3" t="n"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="n"/>
+      <c r="B139" s="3" t="n"/>
+      <c r="C139" s="3" t="n"/>
+      <c r="D139" s="3" t="n"/>
+      <c r="E139" s="3" t="n"/>
+      <c r="F139" s="4" t="n"/>
+      <c r="G139" s="4" t="n"/>
+      <c r="H139" s="4" t="n"/>
+      <c r="I139" s="4" t="n"/>
+      <c r="J139" s="3" t="n"/>
+      <c r="K139" s="2" t="n"/>
+      <c r="L139" s="3" t="n"/>
+      <c r="M139" s="3" t="n"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="n"/>
+      <c r="B140" s="3" t="n"/>
+      <c r="C140" s="3" t="n"/>
+      <c r="D140" s="3" t="n"/>
+      <c r="E140" s="3" t="n"/>
+      <c r="F140" s="4" t="n"/>
+      <c r="G140" s="4" t="n"/>
+      <c r="H140" s="4" t="n"/>
+      <c r="I140" s="4" t="n"/>
+      <c r="J140" s="3" t="n"/>
+      <c r="K140" s="2" t="n"/>
+      <c r="L140" s="3" t="n"/>
+      <c r="M140" s="3" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M90"/>
+  <autoFilter ref="A1:M140"/>
   <conditionalFormatting sqref="A2:M90">
     <cfRule type="expression" priority="2" dxfId="0">
       <formula>$L2="No"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="5">
-    <dataValidation sqref="J2:J90" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="L2:L90" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L2:L140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E90" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Single,Tiered"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K90" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,Partly,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="B2:B90" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B2:B140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Chapters!$A$2:$A$10</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Ledger: the user's sheet edits, and numbered events now stamp
Beginner's Luck is a pet within the day's first 10 Scatha kills (counted from
local midnight); Dentist is 25/50/200/500; Double Haunting is 30 seconds,
Poltergeist and Matched Pair a minute. The Chapter dropdown the scripted save
dropped is back.

Fixed: an awarded event read as 1, so a numbered one (Back to Back 50, In the
Black 30M) was flagged but never stamped. It now reads as its own number.
LedgerTest 409.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E2z82eUcdf81sbDmiwVwoi
</commit_message>
<xml_diff>
--- a/docs/ledger_stamps.xlsx
+++ b/docs/ledger_stamps.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stamps" sheetId="1" state="visible" r:id="rId1"/>
@@ -933,7 +933,7 @@
       </c>
       <c r="M10" s="3" t="n"/>
     </row>
-    <row r="11">
+    <row r="11" ht="28.5" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>house_well_done</t>
@@ -992,7 +992,7 @@
         </is>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="28.5" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>house_collector</t>
@@ -1051,7 +1051,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="28.5" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>house_big_ticket</t>
@@ -1345,7 +1345,7 @@
       </c>
       <c r="M18" s="3" t="n"/>
     </row>
-    <row r="19">
+    <row r="19" ht="42.75" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
           <t>scatha_beginners_luck</t>
@@ -1363,7 +1363,7 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>A pet within your first N kills</t>
+          <t>A pet within your first N kills of the day</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
@@ -1372,7 +1372,7 @@
         </is>
       </c>
       <c r="F19" s="4" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="G19" s="4" t="n"/>
       <c r="H19" s="4" t="n"/>
@@ -1384,7 +1384,7 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Partly</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L19" s="3" t="inlineStr">
@@ -1392,7 +1392,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="M19" s="3" t="n"/>
+      <c r="M19" s="3" t="inlineStr">
+        <is>
+          <t>make it so that it resets every day so its not impossible to get after reaching the number of kills | Claude, 2026-10-16: done - kills are counted from midnight on your clock; a pet in the first 10 of a day earns it. Old stats cannot show which day a pet came, so it is not backfilled (stamps you already have stay).</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1639,7 +1643,7 @@
       </c>
       <c r="M24" s="3" t="n"/>
     </row>
-    <row r="25">
+    <row r="25" ht="28.5" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
           <t>scatha_cereal</t>
@@ -1894,7 +1898,7 @@
       </c>
       <c r="M29" s="3" t="n"/>
     </row>
-    <row r="30">
+    <row r="30" ht="57" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
           <t>vg_ice_cold</t>
@@ -2043,7 +2047,7 @@
       </c>
       <c r="M32" s="3" t="n"/>
     </row>
-    <row r="33">
+    <row r="33" ht="28.5" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
           <t>vg_skeleton_crew</t>
@@ -2102,7 +2106,7 @@
         </is>
       </c>
     </row>
-    <row r="34">
+    <row r="34" ht="28.5" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
           <t>vg_cold_storage</t>
@@ -2161,7 +2165,7 @@
         </is>
       </c>
     </row>
-    <row r="35">
+    <row r="35" ht="28.5" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
           <t>vg_will_o_wisp</t>
@@ -2212,7 +2216,7 @@
         </is>
       </c>
     </row>
-    <row r="36">
+    <row r="36" ht="28.5" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
           <t>vg_tough_skin</t>
@@ -2263,7 +2267,7 @@
         </is>
       </c>
     </row>
-    <row r="37">
+    <row r="37" ht="28.5" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
           <t>vg_master_key</t>
@@ -2792,7 +2796,7 @@
       </c>
       <c r="M47" s="3" t="n"/>
     </row>
-    <row r="48">
+    <row r="48" ht="28.5" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
         <is>
           <t>diana_shared_custody</t>
@@ -2839,7 +2843,7 @@
       </c>
       <c r="M48" s="3" t="n"/>
     </row>
-    <row r="49">
+    <row r="49" ht="28.5" customHeight="1">
       <c r="A49" s="2" t="inlineStr">
         <is>
           <t>diana_inquisition</t>
@@ -3190,7 +3194,7 @@
       </c>
       <c r="M55" s="3" t="n"/>
     </row>
-    <row r="56">
+    <row r="56" ht="28.5" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
         <is>
           <t>hellion_power_trip</t>
@@ -3241,7 +3245,7 @@
         </is>
       </c>
     </row>
-    <row r="57">
+    <row r="57" ht="28.5" customHeight="1">
       <c r="A57" s="2" t="inlineStr">
         <is>
           <t>hellion_cold_feet</t>
@@ -3292,7 +3296,7 @@
         </is>
       </c>
     </row>
-    <row r="58">
+    <row r="58" ht="28.5" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
         <is>
           <t>hellion_blueprints</t>
@@ -3343,7 +3347,7 @@
         </is>
       </c>
     </row>
-    <row r="59">
+    <row r="59" ht="28.5" customHeight="1">
       <c r="A59" s="2" t="inlineStr">
         <is>
           <t>hellion_paragon</t>
@@ -3394,7 +3398,7 @@
         </is>
       </c>
     </row>
-    <row r="60">
+    <row r="60" ht="28.5" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
         <is>
           <t>hellion_hellfire_club</t>
@@ -3453,7 +3457,7 @@
         </is>
       </c>
     </row>
-    <row r="61">
+    <row r="61" ht="28.5" customHeight="1">
       <c r="A61" s="2" t="inlineStr">
         <is>
           <t>hellion_seventh_circle</t>
@@ -3794,7 +3798,7 @@
       </c>
       <c r="M67" s="3" t="n"/>
     </row>
-    <row r="68">
+    <row r="68" ht="28.5" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
         <is>
           <t>lava_thermal_runaway</t>
@@ -3843,7 +3847,7 @@
       </c>
       <c r="M68" s="3" t="n"/>
     </row>
-    <row r="69">
+    <row r="69" ht="28.5" customHeight="1">
       <c r="A69" s="2" t="inlineStr">
         <is>
           <t>lava_chained</t>
@@ -3894,7 +3898,7 @@
         </is>
       </c>
     </row>
-    <row r="70">
+    <row r="70" ht="28.5" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
         <is>
           <t>lava_pinch_me</t>
@@ -3945,7 +3949,7 @@
         </is>
       </c>
     </row>
-    <row r="71">
+    <row r="71" ht="28.5" customHeight="1">
       <c r="A71" s="2" t="inlineStr">
         <is>
           <t>lava_forged</t>
@@ -3996,7 +4000,7 @@
         </is>
       </c>
     </row>
-    <row r="72">
+    <row r="72" ht="28.5" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
         <is>
           <t>lava_shell_shocked</t>
@@ -4047,7 +4051,7 @@
         </is>
       </c>
     </row>
-    <row r="73">
+    <row r="73" ht="28.5" customHeight="1">
       <c r="A73" s="2" t="inlineStr">
         <is>
           <t>lava_hot_catch</t>
@@ -4159,7 +4163,7 @@
       </c>
       <c r="M74" s="3" t="n"/>
     </row>
-    <row r="75">
+    <row r="75" ht="57" customHeight="1">
       <c r="A75" s="2" t="inlineStr">
         <is>
           <t>fin_big_fish</t>
@@ -4353,7 +4357,7 @@
       </c>
       <c r="M78" s="3" t="n"/>
     </row>
-    <row r="79">
+    <row r="79" ht="28.5" customHeight="1">
       <c r="A79" s="2" t="inlineStr">
         <is>
           <t>fin_dentist</t>
@@ -4380,16 +4384,16 @@
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="G79" s="4" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="H79" s="4" t="n">
-        <v>25</v>
+        <v>200</v>
       </c>
       <c r="I79" s="4" t="n">
-        <v>50</v>
+        <v>500</v>
       </c>
       <c r="J79" s="3" t="inlineStr">
         <is>
@@ -4412,7 +4416,7 @@
         </is>
       </c>
     </row>
-    <row r="80">
+    <row r="80" ht="28.5" customHeight="1">
       <c r="A80" s="2" t="inlineStr">
         <is>
           <t>fin_school</t>
@@ -4471,7 +4475,7 @@
         </is>
       </c>
     </row>
-    <row r="81">
+    <row r="81" ht="28.5" customHeight="1">
       <c r="A81" s="2" t="inlineStr">
         <is>
           <t>fin_dry_dock</t>
@@ -4530,7 +4534,7 @@
         </is>
       </c>
     </row>
-    <row r="82">
+    <row r="82" ht="28.5" customHeight="1">
       <c r="A82" s="2" t="inlineStr">
         <is>
           <t>fin_feeding_frenzy</t>
@@ -4581,7 +4585,7 @@
         </is>
       </c>
     </row>
-    <row r="83">
+    <row r="83" ht="28.5" customHeight="1">
       <c r="A83" s="2" t="inlineStr">
         <is>
           <t>fin_both_ends</t>
@@ -4779,7 +4783,7 @@
       </c>
       <c r="M86" s="3" t="n"/>
     </row>
-    <row r="87">
+    <row r="87" ht="28.5" customHeight="1">
       <c r="A87" s="2" t="inlineStr">
         <is>
           <t>wisp_drowning</t>
@@ -4838,7 +4842,7 @@
         </is>
       </c>
     </row>
-    <row r="88">
+    <row r="88" ht="28.5" customHeight="1">
       <c r="A88" s="2" t="inlineStr">
         <is>
           <t>wisp_high_voltage</t>
@@ -4897,7 +4901,7 @@
         </is>
       </c>
     </row>
-    <row r="89">
+    <row r="89" ht="28.5" customHeight="1">
       <c r="A89" s="2" t="inlineStr">
         <is>
           <t>wisp_bittersweet</t>
@@ -4948,7 +4952,7 @@
         </is>
       </c>
     </row>
-    <row r="90">
+    <row r="90" ht="28.5" customHeight="1">
       <c r="A90" s="2" t="inlineStr">
         <is>
           <t>wisp_double_haunting</t>
@@ -4966,7 +4970,7 @@
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>Two Ghost drops within 10 minutes</t>
+          <t>Two Ghost drops within 30 seconds</t>
         </is>
       </c>
       <c r="E90" s="3" t="inlineStr">
@@ -4999,7 +5003,7 @@
         </is>
       </c>
     </row>
-    <row r="91">
+    <row r="91" ht="28.5" customHeight="1">
       <c r="A91" s="2" t="inlineStr">
         <is>
           <t>wisp_poltergeist</t>
@@ -5017,7 +5021,7 @@
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>Three Ghost drops within an hour</t>
+          <t>Three Ghost drops within a minute</t>
         </is>
       </c>
       <c r="E91" s="3" t="inlineStr">
@@ -5050,7 +5054,7 @@
         </is>
       </c>
     </row>
-    <row r="92">
+    <row r="92" ht="28.5" customHeight="1">
       <c r="A92" s="2" t="inlineStr">
         <is>
           <t>wisp_matched_pair</t>
@@ -5068,7 +5072,7 @@
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>Sorrow and Plasma within an hour of each other</t>
+          <t>Sorrow and Plasma within a minute of each other</t>
         </is>
       </c>
       <c r="E92" s="3" t="inlineStr">
@@ -5101,7 +5105,7 @@
         </is>
       </c>
     </row>
-    <row r="93">
+    <row r="93" ht="28.5" customHeight="1">
       <c r="A93" s="2" t="inlineStr">
         <is>
           <t>wisp_witching_hour</t>
@@ -5864,11 +5868,8 @@
       <formula>$L2="No"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="5">
-    <dataValidation sqref="J2:J140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Yes,No"</formula1>
-    </dataValidation>
-    <dataValidation sqref="L2:L140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <dataValidations count="4">
+    <dataValidation sqref="J2:J140 L2:L140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>

<commit_message>
Ledger: 17 new secret stamps with hints, SkyBlock item icons
Secret stamps go from 6 to 27: 17 new event stamps (dates, runs of luck, Cereal Killer, Snake Eyes, Number of the
Beast, Health Inspector...) and four existing ones made secret. Every secret stamp has a pencilled hint from the
sheet's new Hint column; the pop-up says SECRET STAMP!. Regular and Collector renamed.

Stamps for a drop now draw the SkyBlock item from the bundled NEU skins as a skinned player head; the remaining
vanilla stand-ins are listed in docs/TODO.md. LedgerTest 530.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E2z82eUcdf81sbDmiwVwoi
</commit_message>
<xml_diff>
--- a/docs/ledger_stamps.xlsx
+++ b/docs/ledger_stamps.xlsx
@@ -407,7 +407,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M140"/>
+  <dimension ref="A1:N140"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -421,6 +421,7 @@
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="8" customWidth="1" min="12" max="12"/>
     <col width="40" customWidth="1" min="13" max="13"/>
+    <col width="44" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -487,6 +488,11 @@
       <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Your notes</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Hint (secret stamps)</t>
         </is>
       </c>
     </row>
@@ -550,7 +556,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Regular</t>
+          <t>Regular Customer</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -590,7 +596,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="M3" s="3" t="n"/>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-17: renamed from 'Regular' to be a bit funnier.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -720,7 +730,7 @@
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -733,7 +743,16 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="M6" s="3" t="n"/>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-17: made secret (you asked for more).</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Lightning does strike twice.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -885,6 +904,11 @@
         </is>
       </c>
       <c r="M9" s="3" t="n"/>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>The butcher keeps strange hours.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -932,6 +956,11 @@
         </is>
       </c>
       <c r="M10" s="3" t="n"/>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Slot machines love this number.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="28.5" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -1005,7 +1034,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Collector</t>
+          <t>Mixed Grill</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -1047,7 +1076,7 @@
       </c>
       <c r="M12" s="3" t="inlineStr">
         <is>
-          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No. | Claude, 2026-10-17: renamed from 'Collector' to be a bit funnier.</t>
         </is>
       </c>
     </row>
@@ -1495,6 +1524,11 @@
         </is>
       </c>
       <c r="M21" s="3" t="n"/>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Some cuts need a lot longer.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1579,7 +1613,7 @@
       <c r="I23" s="4" t="n"/>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -1592,7 +1626,16 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="M23" s="3" t="n"/>
+      <c r="M23" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-17: made secret (you asked for more).</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Worms come in pairs.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1983,7 +2026,7 @@
       <c r="I31" s="4" t="n"/>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
@@ -1996,7 +2039,16 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="M31" s="3" t="n"/>
+      <c r="M31" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-17: made secret (you asked for more).</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>You paid how much for that key?</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2842,6 +2894,11 @@
         </is>
       </c>
       <c r="M48" s="3" t="n"/>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>Sharing is caring.</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="28.5" customHeight="1">
       <c r="A49" s="2" t="inlineStr">
@@ -3507,6 +3564,11 @@
           <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
         </is>
       </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>Collect the whole set of sins.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -4984,7 +5046,7 @@
       <c r="I90" s="4" t="n"/>
       <c r="J90" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K90" s="2" t="inlineStr">
@@ -4999,7 +5061,12 @@
       </c>
       <c r="M90" s="3" t="inlineStr">
         <is>
-          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
+          <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No. | Claude, 2026-10-17: made secret (you asked for more).</t>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>Twice the boo.</t>
         </is>
       </c>
     </row>
@@ -5155,261 +5222,973 @@
           <t>Claude, 2026-10-16: new, for 10+ a chapter. Edit or set Keep? to No.</t>
         </is>
       </c>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t>Ghosts keep late hours.</t>
+        </is>
+      </c>
     </row>
     <row r="94">
-      <c r="A94" s="2" t="n"/>
-      <c r="B94" s="3" t="n"/>
-      <c r="C94" s="3" t="n"/>
-      <c r="D94" s="3" t="n"/>
-      <c r="E94" s="3" t="n"/>
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>house_unlucky_13</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>House</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>Unlucky for Some</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>A rare drop on a Friday the 13th</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
       <c r="F94" s="4" t="n"/>
       <c r="G94" s="4" t="n"/>
       <c r="H94" s="4" t="n"/>
       <c r="I94" s="4" t="n"/>
-      <c r="J94" s="3" t="n"/>
-      <c r="K94" s="2" t="n"/>
-      <c r="L94" s="3" t="n"/>
-      <c r="M94" s="3" t="n"/>
+      <c r="J94" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K94" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L94" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M94" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-17: new secret stamp. Edit or set Keep? to No.</t>
+        </is>
+      </c>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>Walk under a ladder first.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
-      <c r="A95" s="2" t="n"/>
-      <c r="B95" s="3" t="n"/>
-      <c r="C95" s="3" t="n"/>
-      <c r="D95" s="3" t="n"/>
-      <c r="E95" s="3" t="n"/>
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>house_leap_of_faith</t>
+        </is>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>House</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>Leap of Faith</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>A rare drop on the 29th of February</t>
+        </is>
+      </c>
+      <c r="E95" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
       <c r="F95" s="4" t="n"/>
       <c r="G95" s="4" t="n"/>
       <c r="H95" s="4" t="n"/>
       <c r="I95" s="4" t="n"/>
-      <c r="J95" s="3" t="n"/>
-      <c r="K95" s="2" t="n"/>
-      <c r="L95" s="3" t="n"/>
-      <c r="M95" s="3" t="n"/>
+      <c r="J95" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K95" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L95" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M95" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-17: new secret stamp. Edit or set Keep? to No.</t>
+        </is>
+      </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>Only comes round every four years.</t>
+        </is>
+      </c>
     </row>
     <row r="96">
-      <c r="A96" s="2" t="n"/>
-      <c r="B96" s="3" t="n"/>
-      <c r="C96" s="3" t="n"/>
-      <c r="D96" s="3" t="n"/>
-      <c r="E96" s="3" t="n"/>
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>house_christmas_ham</t>
+        </is>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>House</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>Christmas Ham</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>A rare drop on Christmas Day</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
       <c r="F96" s="4" t="n"/>
       <c r="G96" s="4" t="n"/>
       <c r="H96" s="4" t="n"/>
       <c r="I96" s="4" t="n"/>
-      <c r="J96" s="3" t="n"/>
-      <c r="K96" s="2" t="n"/>
-      <c r="L96" s="3" t="n"/>
-      <c r="M96" s="3" t="n"/>
+      <c r="J96" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K96" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L96" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M96" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-17: new secret stamp. Edit or set Keep? to No.</t>
+        </is>
+      </c>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>Someone was nice this year.</t>
+        </is>
+      </c>
     </row>
     <row r="97">
-      <c r="A97" s="2" t="n"/>
-      <c r="B97" s="3" t="n"/>
-      <c r="C97" s="3" t="n"/>
-      <c r="D97" s="3" t="n"/>
-      <c r="E97" s="3" t="n"/>
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>house_two_timer</t>
+        </is>
+      </c>
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>House</t>
+        </is>
+      </c>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>Two-Timer</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>Rare drops from two different animations within 5 minutes</t>
+        </is>
+      </c>
+      <c r="E97" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
       <c r="F97" s="4" t="n"/>
       <c r="G97" s="4" t="n"/>
       <c r="H97" s="4" t="n"/>
       <c r="I97" s="4" t="n"/>
-      <c r="J97" s="3" t="n"/>
-      <c r="K97" s="2" t="n"/>
-      <c r="L97" s="3" t="n"/>
-      <c r="M97" s="3" t="n"/>
+      <c r="J97" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K97" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L97" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M97" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-17: new secret stamp. Edit or set Keep? to No.</t>
+        </is>
+      </c>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>Why settle for one?</t>
+        </is>
+      </c>
     </row>
     <row r="98">
-      <c r="A98" s="2" t="n"/>
-      <c r="B98" s="3" t="n"/>
-      <c r="C98" s="3" t="n"/>
-      <c r="D98" s="3" t="n"/>
-      <c r="E98" s="3" t="n"/>
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>house_health_inspector</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>House</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>Health Inspector</t>
+        </is>
+      </c>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>Shut a cutscene down with /butcher stop</t>
+        </is>
+      </c>
+      <c r="E98" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
       <c r="F98" s="4" t="n"/>
       <c r="G98" s="4" t="n"/>
       <c r="H98" s="4" t="n"/>
       <c r="I98" s="4" t="n"/>
-      <c r="J98" s="3" t="n"/>
-      <c r="K98" s="2" t="n"/>
-      <c r="L98" s="3" t="n"/>
-      <c r="M98" s="3" t="n"/>
+      <c r="J98" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K98" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L98" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M98" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-17: new secret stamp. Edit or set Keep? to No.</t>
+        </is>
+      </c>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>Close the kitchen.</t>
+        </is>
+      </c>
     </row>
     <row r="99">
-      <c r="A99" s="2" t="n"/>
-      <c r="B99" s="3" t="n"/>
-      <c r="C99" s="3" t="n"/>
-      <c r="D99" s="3" t="n"/>
-      <c r="E99" s="3" t="n"/>
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>house_natural</t>
+        </is>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
+        <is>
+          <t>House</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>Natural Talent</t>
+        </is>
+      </c>
+      <c r="D99" s="3" t="inlineStr">
+        <is>
+          <t>A rare drop on your very first kill for an animation</t>
+        </is>
+      </c>
+      <c r="E99" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
       <c r="F99" s="4" t="n"/>
       <c r="G99" s="4" t="n"/>
       <c r="H99" s="4" t="n"/>
       <c r="I99" s="4" t="n"/>
-      <c r="J99" s="3" t="n"/>
-      <c r="K99" s="2" t="n"/>
-      <c r="L99" s="3" t="n"/>
-      <c r="M99" s="3" t="n"/>
+      <c r="J99" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K99" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L99" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M99" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-17: new secret stamp. Edit or set Keep? to No.</t>
+        </is>
+      </c>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t>First try. Obviously.</t>
+        </is>
+      </c>
     </row>
     <row r="100">
-      <c r="A100" s="2" t="n"/>
-      <c r="B100" s="3" t="n"/>
-      <c r="C100" s="3" t="n"/>
-      <c r="D100" s="3" t="n"/>
-      <c r="E100" s="3" t="n"/>
-      <c r="F100" s="4" t="n"/>
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>house_loose_change</t>
+        </is>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>House</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>Loose Change</t>
+        </is>
+      </c>
+      <c r="D100" s="3" t="inlineStr">
+        <is>
+          <t>A drop revealed worth less than N coins</t>
+        </is>
+      </c>
+      <c r="E100" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="F100" s="4" t="n">
+        <v>500000</v>
+      </c>
       <c r="G100" s="4" t="n"/>
       <c r="H100" s="4" t="n"/>
       <c r="I100" s="4" t="n"/>
-      <c r="J100" s="3" t="n"/>
-      <c r="K100" s="2" t="n"/>
-      <c r="L100" s="3" t="n"/>
-      <c r="M100" s="3" t="n"/>
+      <c r="J100" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K100" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L100" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M100" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-17: new secret stamp. Edit or set Keep? to No.</t>
+        </is>
+      </c>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t>Not every drop pays the rent.</t>
+        </is>
+      </c>
     </row>
     <row r="101">
-      <c r="A101" s="2" t="n"/>
-      <c r="B101" s="3" t="n"/>
-      <c r="C101" s="3" t="n"/>
-      <c r="D101" s="3" t="n"/>
-      <c r="E101" s="3" t="n"/>
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>scatha_round_number</t>
+        </is>
+      </c>
+      <c r="B101" s="3" t="inlineStr">
+        <is>
+          <t>Scatha</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>Round Number</t>
+        </is>
+      </c>
+      <c r="D101" s="3" t="inlineStr">
+        <is>
+          <t>A pet on a Scatha kill that ends in 00</t>
+        </is>
+      </c>
+      <c r="E101" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
       <c r="F101" s="4" t="n"/>
       <c r="G101" s="4" t="n"/>
       <c r="H101" s="4" t="n"/>
       <c r="I101" s="4" t="n"/>
-      <c r="J101" s="3" t="n"/>
-      <c r="K101" s="2" t="n"/>
-      <c r="L101" s="3" t="n"/>
-      <c r="M101" s="3" t="n"/>
+      <c r="J101" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K101" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L101" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M101" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-17: new secret stamp. Edit or set Keep? to No.</t>
+        </is>
+      </c>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t>Nice and tidy.</t>
+        </is>
+      </c>
     </row>
     <row r="102">
-      <c r="A102" s="2" t="n"/>
-      <c r="B102" s="3" t="n"/>
-      <c r="C102" s="3" t="n"/>
-      <c r="D102" s="3" t="n"/>
-      <c r="E102" s="3" t="n"/>
-      <c r="F102" s="4" t="n"/>
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>scatha_is_that_it</t>
+        </is>
+      </c>
+      <c r="B102" s="3" t="inlineStr">
+        <is>
+          <t>Scatha</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>Is That It?</t>
+        </is>
+      </c>
+      <c r="D102" s="3" t="inlineStr">
+        <is>
+          <t>A rare (blue) pet after N kills or more without one</t>
+        </is>
+      </c>
+      <c r="E102" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="F102" s="4" t="n">
+        <v>300</v>
+      </c>
       <c r="G102" s="4" t="n"/>
       <c r="H102" s="4" t="n"/>
       <c r="I102" s="4" t="n"/>
-      <c r="J102" s="3" t="n"/>
-      <c r="K102" s="2" t="n"/>
-      <c r="L102" s="3" t="n"/>
-      <c r="M102" s="3" t="n"/>
+      <c r="J102" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K102" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L102" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M102" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-17: new secret stamp. Edit or set Keep? to No.</t>
+        </is>
+      </c>
+      <c r="N102" t="inlineStr">
+        <is>
+          <t>All that waiting, for this?</t>
+        </is>
+      </c>
     </row>
     <row r="103">
-      <c r="A103" s="2" t="n"/>
-      <c r="B103" s="3" t="n"/>
-      <c r="C103" s="3" t="n"/>
-      <c r="D103" s="3" t="n"/>
-      <c r="E103" s="3" t="n"/>
-      <c r="F103" s="4" t="n"/>
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>scatha_cereal_killer</t>
+        </is>
+      </c>
+      <c r="B103" s="3" t="inlineStr">
+        <is>
+          <t>Scatha</t>
+        </is>
+      </c>
+      <c r="C103" s="3" t="inlineStr">
+        <is>
+          <t>Cereal Killer</t>
+        </is>
+      </c>
+      <c r="D103" s="3" t="inlineStr">
+        <is>
+          <t>N Dwarven O's busts in a row</t>
+        </is>
+      </c>
+      <c r="E103" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="F103" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="G103" s="4" t="n"/>
       <c r="H103" s="4" t="n"/>
       <c r="I103" s="4" t="n"/>
-      <c r="J103" s="3" t="n"/>
-      <c r="K103" s="2" t="n"/>
-      <c r="L103" s="3" t="n"/>
-      <c r="M103" s="3" t="n"/>
+      <c r="J103" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K103" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L103" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M103" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-17: new secret stamp. Edit or set Keep? to No.</t>
+        </is>
+      </c>
+      <c r="N103" t="inlineStr">
+        <is>
+          <t>An unbalanced breakfast.</t>
+        </is>
+      </c>
     </row>
     <row r="104">
-      <c r="A104" s="2" t="n"/>
-      <c r="B104" s="3" t="n"/>
-      <c r="C104" s="3" t="n"/>
-      <c r="D104" s="3" t="n"/>
-      <c r="E104" s="3" t="n"/>
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>vg_brain_freeze</t>
+        </is>
+      </c>
+      <c r="B104" s="3" t="inlineStr">
+        <is>
+          <t>Vanguard</t>
+        </is>
+      </c>
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>Brain Freeze</t>
+        </is>
+      </c>
+      <c r="D104" s="3" t="inlineStr">
+        <is>
+          <t>Two legendaries (or better) out of one corpse</t>
+        </is>
+      </c>
+      <c r="E104" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
       <c r="F104" s="4" t="n"/>
       <c r="G104" s="4" t="n"/>
       <c r="H104" s="4" t="n"/>
       <c r="I104" s="4" t="n"/>
-      <c r="J104" s="3" t="n"/>
-      <c r="K104" s="2" t="n"/>
-      <c r="L104" s="3" t="n"/>
-      <c r="M104" s="3" t="n"/>
+      <c r="J104" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K104" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L104" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M104" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-17: new secret stamp. Edit or set Keep? to No.</t>
+        </is>
+      </c>
+      <c r="N104" t="inlineStr">
+        <is>
+          <t>One scoop is never enough.</t>
+        </is>
+      </c>
     </row>
     <row r="105">
-      <c r="A105" s="2" t="n"/>
-      <c r="B105" s="3" t="n"/>
-      <c r="C105" s="3" t="n"/>
-      <c r="D105" s="3" t="n"/>
-      <c r="E105" s="3" t="n"/>
-      <c r="F105" s="4" t="n"/>
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>diana_nobody_expects</t>
+        </is>
+      </c>
+      <c r="B105" s="3" t="inlineStr">
+        <is>
+          <t>Diana</t>
+        </is>
+      </c>
+      <c r="C105" s="3" t="inlineStr">
+        <is>
+          <t>Nobody Expects It</t>
+        </is>
+      </c>
+      <c r="D105" s="3" t="inlineStr">
+        <is>
+          <t>A rare drop within your first N Minos Inquisitor kills</t>
+        </is>
+      </c>
+      <c r="E105" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="F105" s="4" t="n">
+        <v>10</v>
+      </c>
       <c r="G105" s="4" t="n"/>
       <c r="H105" s="4" t="n"/>
       <c r="I105" s="4" t="n"/>
-      <c r="J105" s="3" t="n"/>
-      <c r="K105" s="2" t="n"/>
-      <c r="L105" s="3" t="n"/>
-      <c r="M105" s="3" t="n"/>
+      <c r="J105" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K105" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L105" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M105" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-17: new secret stamp. Edit or set Keep? to No.</t>
+        </is>
+      </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>Its chief weapon is surprise.</t>
+        </is>
+      </c>
     </row>
     <row r="106">
-      <c r="A106" s="2" t="n"/>
-      <c r="B106" s="3" t="n"/>
-      <c r="C106" s="3" t="n"/>
-      <c r="D106" s="3" t="n"/>
-      <c r="E106" s="3" t="n"/>
-      <c r="F106" s="4" t="n"/>
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>hellion_number_beast</t>
+        </is>
+      </c>
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>Hellion</t>
+        </is>
+      </c>
+      <c r="C106" s="3" t="inlineStr">
+        <is>
+          <t>Number of the Beast</t>
+        </is>
+      </c>
+      <c r="D106" s="3" t="inlineStr">
+        <is>
+          <t>A Demonlord drop on exactly your Nth Demonlord kill</t>
+        </is>
+      </c>
+      <c r="E106" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="F106" s="4" t="n">
+        <v>666</v>
+      </c>
       <c r="G106" s="4" t="n"/>
       <c r="H106" s="4" t="n"/>
       <c r="I106" s="4" t="n"/>
-      <c r="J106" s="3" t="n"/>
-      <c r="K106" s="2" t="n"/>
-      <c r="L106" s="3" t="n"/>
-      <c r="M106" s="3" t="n"/>
+      <c r="J106" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K106" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L106" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M106" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-17: new secret stamp. Edit or set Keep? to No.</t>
+        </is>
+      </c>
+      <c r="N106" t="inlineStr">
+        <is>
+          <t>Devilishly specific.</t>
+        </is>
+      </c>
     </row>
     <row r="107">
-      <c r="A107" s="2" t="n"/>
-      <c r="B107" s="3" t="n"/>
-      <c r="C107" s="3" t="n"/>
-      <c r="D107" s="3" t="n"/>
-      <c r="E107" s="3" t="n"/>
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>hellion_snake_eyes</t>
+        </is>
+      </c>
+      <c r="B107" s="3" t="inlineStr">
+        <is>
+          <t>Hellion</t>
+        </is>
+      </c>
+      <c r="C107" s="3" t="inlineStr">
+        <is>
+          <t>Snake Eyes</t>
+        </is>
+      </c>
+      <c r="D107" s="3" t="inlineStr">
+        <is>
+          <t>Archfiend Dice from two Demonlord drops in a row</t>
+        </is>
+      </c>
+      <c r="E107" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
       <c r="F107" s="4" t="n"/>
       <c r="G107" s="4" t="n"/>
       <c r="H107" s="4" t="n"/>
       <c r="I107" s="4" t="n"/>
-      <c r="J107" s="3" t="n"/>
-      <c r="K107" s="2" t="n"/>
-      <c r="L107" s="3" t="n"/>
-      <c r="M107" s="3" t="n"/>
+      <c r="J107" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K107" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L107" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M107" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-17: new secret stamp. Edit or set Keep? to No.</t>
+        </is>
+      </c>
+      <c r="N107" t="inlineStr">
+        <is>
+          <t>Roll again.</t>
+        </is>
+      </c>
     </row>
     <row r="108">
-      <c r="A108" s="2" t="n"/>
-      <c r="B108" s="3" t="n"/>
-      <c r="C108" s="3" t="n"/>
-      <c r="D108" s="3" t="n"/>
-      <c r="E108" s="3" t="n"/>
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>lava_hot_potato</t>
+        </is>
+      </c>
+      <c r="B108" s="3" t="inlineStr">
+        <is>
+          <t>Eruption</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>Hot Potato</t>
+        </is>
+      </c>
+      <c r="D108" s="3" t="inlineStr">
+        <is>
+          <t>Two lava creature drops within 5 minutes</t>
+        </is>
+      </c>
+      <c r="E108" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
       <c r="F108" s="4" t="n"/>
       <c r="G108" s="4" t="n"/>
       <c r="H108" s="4" t="n"/>
       <c r="I108" s="4" t="n"/>
-      <c r="J108" s="3" t="n"/>
-      <c r="K108" s="2" t="n"/>
-      <c r="L108" s="3" t="n"/>
-      <c r="M108" s="3" t="n"/>
+      <c r="J108" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K108" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L108" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M108" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-17: new secret stamp. Edit or set Keep? to No.</t>
+        </is>
+      </c>
+      <c r="N108" t="inlineStr">
+        <is>
+          <t>Too hot to hold.</t>
+        </is>
+      </c>
     </row>
     <row r="109">
-      <c r="A109" s="2" t="n"/>
-      <c r="B109" s="3" t="n"/>
-      <c r="C109" s="3" t="n"/>
-      <c r="D109" s="3" t="n"/>
-      <c r="E109" s="3" t="n"/>
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>fin_bigger_boat</t>
+        </is>
+      </c>
+      <c r="B109" s="3" t="inlineStr">
+        <is>
+          <t>Fin</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>Gonna Need a Bigger Boat</t>
+        </is>
+      </c>
+      <c r="D109" s="3" t="inlineStr">
+        <is>
+          <t>Three shark drops within 10 minutes</t>
+        </is>
+      </c>
+      <c r="E109" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
       <c r="F109" s="4" t="n"/>
       <c r="G109" s="4" t="n"/>
       <c r="H109" s="4" t="n"/>
       <c r="I109" s="4" t="n"/>
-      <c r="J109" s="3" t="n"/>
-      <c r="K109" s="2" t="n"/>
-      <c r="L109" s="3" t="n"/>
-      <c r="M109" s="3" t="n"/>
+      <c r="J109" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K109" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L109" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M109" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-17: new secret stamp. Edit or set Keep? to No.</t>
+        </is>
+      </c>
+      <c r="N109" t="inlineStr">
+        <is>
+          <t>Bring something larger.</t>
+        </is>
+      </c>
     </row>
     <row r="110">
-      <c r="A110" s="2" t="n"/>
-      <c r="B110" s="3" t="n"/>
-      <c r="C110" s="3" t="n"/>
-      <c r="D110" s="3" t="n"/>
-      <c r="E110" s="3" t="n"/>
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>wisp_aint_afraid</t>
+        </is>
+      </c>
+      <c r="B110" s="3" t="inlineStr">
+        <is>
+          <t>Wisp</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>Ain't Afraid of No Ghost</t>
+        </is>
+      </c>
+      <c r="D110" s="3" t="inlineStr">
+        <is>
+          <t>Five Ghost drops within 10 minutes</t>
+        </is>
+      </c>
+      <c r="E110" s="3" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
       <c r="F110" s="4" t="n"/>
       <c r="G110" s="4" t="n"/>
       <c r="H110" s="4" t="n"/>
       <c r="I110" s="4" t="n"/>
-      <c r="J110" s="3" t="n"/>
-      <c r="K110" s="2" t="n"/>
-      <c r="L110" s="3" t="n"/>
-      <c r="M110" s="3" t="n"/>
+      <c r="J110" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K110" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L110" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M110" s="3" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-17: new secret stamp. Edit or set Keep? to No.</t>
+        </is>
+      </c>
+      <c r="N110" t="inlineStr">
+        <is>
+          <t>Who you gonna call?</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n"/>
@@ -5893,7 +6672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -5976,48 +6755,55 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="n"/>
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Hint           Secret stamps only: a pencilled clue shown in place of the rule until it is earned.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="6" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>Do not change the ID column: it is how I match your edits to the code. New stamps get a new ID.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>To add a stamp, fill in a new row at the bottom, for example:</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
+          <t>To add a stamp, fill in a new row at the bottom, for example:</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">  ID: scatha_unlucky_13 | Chapter: Scatha | Stamp name: Thirteen | What earns it: A pet on your 13th kill of the day | Kind: Single | Hidden?: Yes | Keep?: Yes</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="6" t="n"/>
-    </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>Backfill (grey, mine to fill): whether your existing stats can award it on the update - Yes, Partly, or No (starts counting from the update).</t>
-        </is>
-      </c>
+      <c r="A18" s="6" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Decisions sheet: the open questions for the whole Ledger.</t>
+          <t>Backfill (grey, mine to fill): whether your existing stats can award it on the update - Yes, Partly, or No (starts counting from the update).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Decisions sheet: the open questions for the whole Ledger.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>Chapters sheet: counts per chapter, worked out from the Stamps sheet.</t>
         </is>

</xml_diff>

<commit_message>
Ledger: no text lines round the book; Natural Talent and Nobody Expects It reset daily
The "Back to the menu" link and the hint line are gone (Esc and the ribbon still close it), and the book takes the
room. Natural Talent is a drop on the day's first kill of an animation, Nobody Expects It a drop within the day's
first 5 Inquisitors: Ledger.kill keeps per-animation counts for the local day. LedgerTest 535.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E2z82eUcdf81sbDmiwVwoi
</commit_message>
<xml_diff>
--- a/docs/ledger_stamps.xlsx
+++ b/docs/ledger_stamps.xlsx
@@ -5526,7 +5526,7 @@
       </c>
       <c r="D99" s="3" t="inlineStr">
         <is>
-          <t>A rare drop on your very first kill for an animation</t>
+          <t>A rare drop on the day's first kill for an animation</t>
         </is>
       </c>
       <c r="E99" s="3" t="inlineStr">
@@ -5555,7 +5555,7 @@
       </c>
       <c r="M99" s="3" t="inlineStr">
         <is>
-          <t>Claude, 2026-10-17: new secret stamp. Edit or set Keep? to No.</t>
+          <t>Claude, 2026-10-17: new secret stamp. Edit or set Keep? to No. | Claude, 2026-10-17: resets every day (your ask).</t>
         </is>
       </c>
       <c r="N99" t="inlineStr">
@@ -5868,7 +5868,7 @@
       </c>
       <c r="D105" s="3" t="inlineStr">
         <is>
-          <t>A rare drop within your first N Minos Inquisitor kills</t>
+          <t>A rare drop within your first N Minos Inquisitor kills of the day</t>
         </is>
       </c>
       <c r="E105" s="3" t="inlineStr">
@@ -5877,7 +5877,7 @@
         </is>
       </c>
       <c r="F105" s="4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G105" s="4" t="n"/>
       <c r="H105" s="4" t="n"/>
@@ -5899,7 +5899,7 @@
       </c>
       <c r="M105" s="3" t="inlineStr">
         <is>
-          <t>Claude, 2026-10-17: new secret stamp. Edit or set Keep? to No.</t>
+          <t>Claude, 2026-10-17: new secret stamp. Edit or set Keep? to No. | Claude, 2026-10-17: resets every day (your ask), 5 Inquisitors.</t>
         </is>
       </c>
       <c r="N105" t="inlineStr">

</xml_diff>